<commit_message>
chore(dst): refresh REQ-17-D01 daily-sales outputs (automation regen)
Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/development/abiraj_mini_aios_workbench/projects/PRJ-2026-015_daily-sales-track/evidence/final_outputs/REQ-17_daily-sales-track/REQ-17-D01_daily_sales_track.xlsx
+++ b/development/abiraj_mini_aios_workbench/projects/PRJ-2026-015_daily-sales-track/evidence/final_outputs/REQ-17_daily-sales-track/REQ-17-D01_daily_sales_track.xlsx
@@ -657,13 +657,13 @@
         </is>
       </c>
       <c r="D2" s="3" t="n">
-        <v>46236</v>
+        <v>46237</v>
       </c>
       <c r="E2" s="4" t="n">
+        <v>1522.4</v>
+      </c>
+      <c r="F2" s="4" t="n">
         <v>1128.69</v>
-      </c>
-      <c r="F2" s="4" t="n">
-        <v>932.88</v>
       </c>
       <c r="G2" s="4">
         <f>E2-F2</f>
@@ -674,36 +674,36 @@
         <v/>
       </c>
       <c r="I2" s="4" t="n">
-        <v>1070.98</v>
+        <v>1445.52</v>
       </c>
       <c r="J2" s="6" t="n">
+        <v>65</v>
+      </c>
+      <c r="K2" s="6" t="n">
         <v>64</v>
-      </c>
-      <c r="K2" s="6" t="n">
-        <v>53</v>
       </c>
       <c r="L2" s="5">
         <f>IF(K2=0,"",(J2-K2)/K2)</f>
         <v/>
       </c>
       <c r="M2" s="6" t="n">
-        <v>74</v>
+        <v>69</v>
       </c>
       <c r="N2" s="6" t="n">
-        <v>85</v>
+        <v>126</v>
       </c>
       <c r="O2" s="4">
         <f>IF(J2=0,"",E2/J2)</f>
         <v/>
       </c>
       <c r="P2" s="6" t="n">
-        <v>3036</v>
+        <v>3037</v>
       </c>
       <c r="Q2" s="6" t="n">
-        <v>1731</v>
+        <v>1732</v>
       </c>
       <c r="R2" s="4" t="n">
-        <v>568.36</v>
+        <v>745.54</v>
       </c>
       <c r="S2" s="2">
         <f>IF(AND('Engine Inputs'!E2=0,R2=0),"",IF('Engine Inputs'!E2=0,"📈 Up",IF((R2-'Engine Inputs'!E2)/'Engine Inputs'!E2&gt;Config!$B$2,"📈 Up",IF((R2-'Engine Inputs'!E2)/'Engine Inputs'!E2&lt;-Config!$B$2,"📉 Down","➡ Stable"))))</f>
@@ -713,7 +713,7 @@
         <v>1305</v>
       </c>
       <c r="U2" s="4" t="n">
-        <v>548.76</v>
+        <v>806.4299999999999</v>
       </c>
       <c r="V2" s="2">
         <f>IF(AND('Engine Inputs'!D2=0,U2=0),"",IF('Engine Inputs'!D2=0,"📈 Up",IF((U2-'Engine Inputs'!D2)/'Engine Inputs'!D2&gt;Config!$B$2,"📈 Up",IF((U2-'Engine Inputs'!D2)/'Engine Inputs'!D2&lt;-Config!$B$2,"📉 Down","➡ Stable"))))</f>
@@ -746,13 +746,13 @@
         </is>
       </c>
       <c r="D3" s="3" t="n">
-        <v>46236</v>
+        <v>46237</v>
       </c>
       <c r="E3" s="4" t="n">
+        <v>341.93</v>
+      </c>
+      <c r="F3" s="4" t="n">
         <v>353.49</v>
-      </c>
-      <c r="F3" s="4" t="n">
-        <v>549.5</v>
       </c>
       <c r="G3" s="4">
         <f>E3-F3</f>
@@ -763,36 +763,36 @@
         <v/>
       </c>
       <c r="I3" s="4" t="n">
-        <v>607.8200000000001</v>
+        <v>629.22</v>
       </c>
       <c r="J3" s="6" t="n">
+        <v>23</v>
+      </c>
+      <c r="K3" s="6" t="n">
         <v>21</v>
-      </c>
-      <c r="K3" s="6" t="n">
-        <v>31</v>
       </c>
       <c r="L3" s="5">
         <f>IF(K3=0,"",(J3-K3)/K3)</f>
         <v/>
       </c>
       <c r="M3" s="6" t="n">
-        <v>35</v>
+        <v>37</v>
       </c>
       <c r="N3" s="6" t="n">
-        <v>32</v>
+        <v>26</v>
       </c>
       <c r="O3" s="4">
         <f>IF(J3=0,"",E3/J3)</f>
         <v/>
       </c>
       <c r="P3" s="6" t="n">
-        <v>1678</v>
+        <v>1679</v>
       </c>
       <c r="Q3" s="6" t="n">
-        <v>1081</v>
+        <v>1082</v>
       </c>
       <c r="R3" s="4" t="n">
-        <v>222.27</v>
+        <v>216.66</v>
       </c>
       <c r="S3" s="2">
         <f>IF(AND('Engine Inputs'!E3=0,R3=0),"",IF('Engine Inputs'!E3=0,"📈 Up",IF((R3-'Engine Inputs'!E3)/'Engine Inputs'!E3&gt;Config!$B$2,"📈 Up",IF((R3-'Engine Inputs'!E3)/'Engine Inputs'!E3&lt;-Config!$B$2,"📉 Down","➡ Stable"))))</f>
@@ -802,7 +802,7 @@
         <v>597</v>
       </c>
       <c r="U3" s="4" t="n">
-        <v>147.44</v>
+        <v>128.8</v>
       </c>
       <c r="V3" s="2">
         <f>IF(AND('Engine Inputs'!D3=0,U3=0),"",IF('Engine Inputs'!D3=0,"📈 Up",IF((U3-'Engine Inputs'!D3)/'Engine Inputs'!D3&gt;Config!$B$2,"📈 Up",IF((U3-'Engine Inputs'!D3)/'Engine Inputs'!D3&lt;-Config!$B$2,"📉 Down","➡ Stable"))))</f>
@@ -835,13 +835,13 @@
         </is>
       </c>
       <c r="D4" s="3" t="n">
-        <v>46236</v>
+        <v>46237</v>
       </c>
       <c r="E4" s="7" t="n">
+        <v>393.41</v>
+      </c>
+      <c r="F4" s="7" t="n">
         <v>340.06</v>
-      </c>
-      <c r="F4" s="7" t="n">
-        <v>259.33</v>
       </c>
       <c r="G4" s="7">
         <f>E4-F4</f>
@@ -852,36 +852,36 @@
         <v/>
       </c>
       <c r="I4" s="7" t="n">
-        <v>396.06</v>
+        <v>611.78</v>
       </c>
       <c r="J4" s="6" t="n">
         <v>12</v>
       </c>
       <c r="K4" s="6" t="n">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="L4" s="5">
         <f>IF(K4=0,"",(J4-K4)/K4)</f>
         <v/>
       </c>
       <c r="M4" s="6" t="n">
-        <v>24</v>
+        <v>40</v>
       </c>
       <c r="N4" s="6" t="n">
-        <v>30</v>
+        <v>26</v>
       </c>
       <c r="O4" s="7">
         <f>IF(J4=0,"",E4/J4)</f>
         <v/>
       </c>
       <c r="P4" s="6" t="n">
-        <v>1441</v>
+        <v>1443</v>
       </c>
       <c r="Q4" s="6" t="n">
-        <v>1209</v>
+        <v>1211</v>
       </c>
       <c r="R4" s="7" t="n">
-        <v>273.58</v>
+        <v>315.96</v>
       </c>
       <c r="S4" s="2">
         <f>IF(AND('Engine Inputs'!E4=0,R4=0),"",IF('Engine Inputs'!E4=0,"📈 Up",IF((R4-'Engine Inputs'!E4)/'Engine Inputs'!E4&gt;Config!$B$2,"📈 Up",IF((R4-'Engine Inputs'!E4)/'Engine Inputs'!E4&lt;-Config!$B$2,"📉 Down","➡ Stable"))))</f>
@@ -891,7 +891,7 @@
         <v>232</v>
       </c>
       <c r="U4" s="7" t="n">
-        <v>16.7</v>
+        <v>0</v>
       </c>
       <c r="V4" s="2">
         <f>IF(AND('Engine Inputs'!D4=0,U4=0),"",IF('Engine Inputs'!D4=0,"📈 Up",IF((U4-'Engine Inputs'!D4)/'Engine Inputs'!D4&gt;Config!$B$2,"📈 Up",IF((U4-'Engine Inputs'!D4)/'Engine Inputs'!D4&lt;-Config!$B$2,"📉 Down","➡ Stable"))))</f>
@@ -924,13 +924,13 @@
         </is>
       </c>
       <c r="D5" s="3" t="n">
-        <v>46236</v>
+        <v>46237</v>
       </c>
       <c r="E5" s="4" t="n">
+        <v>126.17</v>
+      </c>
+      <c r="F5" s="4" t="n">
         <v>289.57</v>
-      </c>
-      <c r="F5" s="4" t="n">
-        <v>300.45</v>
       </c>
       <c r="G5" s="4">
         <f>E5-F5</f>
@@ -941,23 +941,23 @@
         <v/>
       </c>
       <c r="I5" s="4" t="n">
-        <v>322.23</v>
+        <v>191.14</v>
       </c>
       <c r="J5" s="6" t="n">
+        <v>9</v>
+      </c>
+      <c r="K5" s="6" t="n">
         <v>16</v>
-      </c>
-      <c r="K5" s="6" t="n">
-        <v>15</v>
       </c>
       <c r="L5" s="5">
         <f>IF(K5=0,"",(J5-K5)/K5)</f>
         <v/>
       </c>
       <c r="M5" s="6" t="n">
-        <v>20</v>
+        <v>11</v>
       </c>
       <c r="N5" s="6" t="n">
-        <v>24</v>
+        <v>10</v>
       </c>
       <c r="O5" s="4">
         <f>IF(J5=0,"",E5/J5)</f>
@@ -970,7 +970,7 @@
         <v>718</v>
       </c>
       <c r="R5" s="4" t="n">
-        <v>206.2</v>
+        <v>98.65000000000001</v>
       </c>
       <c r="S5" s="2">
         <f>IF(AND('Engine Inputs'!E5=0,R5=0),"",IF('Engine Inputs'!E5=0,"📈 Up",IF((R5-'Engine Inputs'!E5)/'Engine Inputs'!E5&gt;Config!$B$2,"📈 Up",IF((R5-'Engine Inputs'!E5)/'Engine Inputs'!E5&lt;-Config!$B$2,"📉 Down","➡ Stable"))))</f>
@@ -980,7 +980,7 @@
         <v>469</v>
       </c>
       <c r="U5" s="4" t="n">
-        <v>78.81</v>
+        <v>24.55</v>
       </c>
       <c r="V5" s="2">
         <f>IF(AND('Engine Inputs'!D5=0,U5=0),"",IF('Engine Inputs'!D5=0,"📈 Up",IF((U5-'Engine Inputs'!D5)/'Engine Inputs'!D5&gt;Config!$B$2,"📈 Up",IF((U5-'Engine Inputs'!D5)/'Engine Inputs'!D5&lt;-Config!$B$2,"📉 Down","➡ Stable"))))</f>
@@ -1013,13 +1013,13 @@
         </is>
       </c>
       <c r="D6" s="3" t="n">
-        <v>46236</v>
+        <v>46237</v>
       </c>
       <c r="E6" s="7" t="n">
+        <v>146.48</v>
+      </c>
+      <c r="F6" s="7" t="n">
         <v>275.07</v>
-      </c>
-      <c r="F6" s="7" t="n">
-        <v>422.04</v>
       </c>
       <c r="G6" s="7">
         <f>E6-F6</f>
@@ -1030,46 +1030,46 @@
         <v/>
       </c>
       <c r="I6" s="7" t="n">
-        <v>273</v>
+        <v>470.64</v>
       </c>
       <c r="J6" s="6" t="n">
+        <v>6</v>
+      </c>
+      <c r="K6" s="6" t="n">
         <v>15</v>
-      </c>
-      <c r="K6" s="6" t="n">
-        <v>10</v>
       </c>
       <c r="L6" s="5">
         <f>IF(K6=0,"",(J6-K6)/K6)</f>
         <v/>
       </c>
       <c r="M6" s="6" t="n">
-        <v>14</v>
+        <v>23</v>
       </c>
       <c r="N6" s="6" t="n">
-        <v>22</v>
+        <v>9</v>
       </c>
       <c r="O6" s="7">
         <f>IF(J6=0,"",E6/J6)</f>
         <v/>
       </c>
       <c r="P6" s="6" t="n">
-        <v>653</v>
+        <v>666</v>
       </c>
       <c r="Q6" s="6" t="n">
-        <v>569</v>
+        <v>577</v>
       </c>
       <c r="R6" s="7" t="n">
-        <v>223.46</v>
+        <v>122.92</v>
       </c>
       <c r="S6" s="2">
         <f>IF(AND('Engine Inputs'!E6=0,R6=0),"",IF('Engine Inputs'!E6=0,"📈 Up",IF((R6-'Engine Inputs'!E6)/'Engine Inputs'!E6&gt;Config!$B$2,"📈 Up",IF((R6-'Engine Inputs'!E6)/'Engine Inputs'!E6&lt;-Config!$B$2,"📉 Down","➡ Stable"))))</f>
         <v/>
       </c>
       <c r="T6" s="6" t="n">
-        <v>84</v>
+        <v>89</v>
       </c>
       <c r="U6" s="7" t="n">
-        <v>48.65</v>
+        <v>0</v>
       </c>
       <c r="V6" s="2">
         <f>IF(AND('Engine Inputs'!D6=0,U6=0),"",IF('Engine Inputs'!D6=0,"📈 Up",IF((U6-'Engine Inputs'!D6)/'Engine Inputs'!D6&gt;Config!$B$2,"📈 Up",IF((U6-'Engine Inputs'!D6)/'Engine Inputs'!D6&lt;-Config!$B$2,"📉 Down","➡ Stable"))))</f>
@@ -1102,7 +1102,7 @@
         </is>
       </c>
       <c r="D7" s="3" t="n">
-        <v>46236</v>
+        <v>46237</v>
       </c>
       <c r="E7" s="7" t="n">
         <v>0</v>
@@ -1191,7 +1191,7 @@
         </is>
       </c>
       <c r="D8" s="3" t="n">
-        <v>46236</v>
+        <v>46237</v>
       </c>
       <c r="E8" s="7" t="n">
         <v>0</v>
@@ -1280,13 +1280,13 @@
         </is>
       </c>
       <c r="D9" s="3" t="n">
-        <v>46236</v>
+        <v>46237</v>
       </c>
       <c r="E9" s="4" t="n">
+        <v>114.14</v>
+      </c>
+      <c r="F9" s="4" t="n">
         <v>189.64</v>
-      </c>
-      <c r="F9" s="4" t="n">
-        <v>256.34</v>
       </c>
       <c r="G9" s="4">
         <f>E9-F9</f>
@@ -1297,23 +1297,23 @@
         <v/>
       </c>
       <c r="I9" s="4" t="n">
-        <v>229.19</v>
+        <v>399.68</v>
       </c>
       <c r="J9" s="6" t="n">
         <v>9</v>
       </c>
       <c r="K9" s="6" t="n">
-        <v>17</v>
+        <v>9</v>
       </c>
       <c r="L9" s="5">
         <f>IF(K9=0,"",(J9-K9)/K9)</f>
         <v/>
       </c>
       <c r="M9" s="6" t="n">
-        <v>16</v>
+        <v>20</v>
       </c>
       <c r="N9" s="6" t="n">
-        <v>11</v>
+        <v>9</v>
       </c>
       <c r="O9" s="4">
         <f>IF(J9=0,"",E9/J9)</f>
@@ -1326,7 +1326,7 @@
         <v>579</v>
       </c>
       <c r="R9" s="4" t="n">
-        <v>186.65</v>
+        <v>108.16</v>
       </c>
       <c r="S9" s="2">
         <f>IF(AND('Engine Inputs'!E9=0,R9=0),"",IF('Engine Inputs'!E9=0,"📈 Up",IF((R9-'Engine Inputs'!E9)/'Engine Inputs'!E9&gt;Config!$B$2,"📈 Up",IF((R9-'Engine Inputs'!E9)/'Engine Inputs'!E9&lt;-Config!$B$2,"📉 Down","➡ Stable"))))</f>
@@ -1369,13 +1369,13 @@
         </is>
       </c>
       <c r="D10" s="3" t="n">
-        <v>46236</v>
+        <v>46237</v>
       </c>
       <c r="E10" s="7" t="n">
+        <v>390.64</v>
+      </c>
+      <c r="F10" s="7" t="n">
         <v>651.92</v>
-      </c>
-      <c r="F10" s="7" t="n">
-        <v>179</v>
       </c>
       <c r="G10" s="7">
         <f>E10-F10</f>
@@ -1386,36 +1386,36 @@
         <v/>
       </c>
       <c r="I10" s="7" t="n">
-        <v>520.39</v>
+        <v>591.05</v>
       </c>
       <c r="J10" s="6" t="n">
+        <v>14</v>
+      </c>
+      <c r="K10" s="6" t="n">
         <v>30</v>
-      </c>
-      <c r="K10" s="6" t="n">
-        <v>10</v>
       </c>
       <c r="L10" s="5">
         <f>IF(K10=0,"",(J10-K10)/K10)</f>
         <v/>
       </c>
       <c r="M10" s="6" t="n">
-        <v>19</v>
+        <v>29</v>
       </c>
       <c r="N10" s="6" t="n">
-        <v>39</v>
+        <v>17</v>
       </c>
       <c r="O10" s="7">
         <f>IF(J10=0,"",E10/J10)</f>
         <v/>
       </c>
       <c r="P10" s="6" t="n">
-        <v>556</v>
+        <v>557</v>
       </c>
       <c r="Q10" s="6" t="n">
-        <v>463</v>
+        <v>464</v>
       </c>
       <c r="R10" s="7" t="n">
-        <v>608.15</v>
+        <v>258.52</v>
       </c>
       <c r="S10" s="2">
         <f>IF(AND('Engine Inputs'!E10=0,R10=0),"",IF('Engine Inputs'!E10=0,"📈 Up",IF((R10-'Engine Inputs'!E10)/'Engine Inputs'!E10&gt;Config!$B$2,"📈 Up",IF((R10-'Engine Inputs'!E10)/'Engine Inputs'!E10&lt;-Config!$B$2,"📉 Down","➡ Stable"))))</f>
@@ -1425,7 +1425,7 @@
         <v>93</v>
       </c>
       <c r="U10" s="7" t="n">
-        <v>47.37</v>
+        <v>63.9</v>
       </c>
       <c r="V10" s="2">
         <f>IF(AND('Engine Inputs'!D10=0,U10=0),"",IF('Engine Inputs'!D10=0,"📈 Up",IF((U10-'Engine Inputs'!D10)/'Engine Inputs'!D10&gt;Config!$B$2,"📈 Up",IF((U10-'Engine Inputs'!D10)/'Engine Inputs'!D10&lt;-Config!$B$2,"📉 Down","➡ Stable"))))</f>
@@ -1458,13 +1458,13 @@
         </is>
       </c>
       <c r="D11" s="3" t="n">
-        <v>46236</v>
+        <v>46237</v>
       </c>
       <c r="E11" s="4" t="n">
+        <v>65.13</v>
+      </c>
+      <c r="F11" s="4" t="n">
         <v>47.85</v>
-      </c>
-      <c r="F11" s="4" t="n">
-        <v>43.83</v>
       </c>
       <c r="G11" s="4">
         <f>E11-F11</f>
@@ -1475,23 +1475,23 @@
         <v/>
       </c>
       <c r="I11" s="4" t="n">
-        <v>98.73</v>
+        <v>67.23</v>
       </c>
       <c r="J11" s="6" t="n">
+        <v>8</v>
+      </c>
+      <c r="K11" s="6" t="n">
         <v>5</v>
-      </c>
-      <c r="K11" s="6" t="n">
-        <v>4</v>
       </c>
       <c r="L11" s="5">
         <f>IF(K11=0,"",(J11-K11)/K11)</f>
         <v/>
       </c>
       <c r="M11" s="6" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="N11" s="6" t="n">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="O11" s="4">
         <f>IF(J11=0,"",E11/J11)</f>
@@ -1504,7 +1504,7 @@
         <v>508</v>
       </c>
       <c r="R11" s="4" t="n">
-        <v>50.29</v>
+        <v>67.40000000000001</v>
       </c>
       <c r="S11" s="2">
         <f>IF(AND('Engine Inputs'!E11=0,R11=0),"",IF('Engine Inputs'!E11=0,"📈 Up",IF((R11-'Engine Inputs'!E11)/'Engine Inputs'!E11&gt;Config!$B$2,"📈 Up",IF((R11-'Engine Inputs'!E11)/'Engine Inputs'!E11&lt;-Config!$B$2,"📉 Down","➡ Stable"))))</f>
@@ -1547,13 +1547,13 @@
         </is>
       </c>
       <c r="D12" s="3" t="n">
-        <v>46236</v>
+        <v>46237</v>
       </c>
       <c r="E12" s="7" t="n">
+        <v>42.87</v>
+      </c>
+      <c r="F12" s="7" t="n">
         <v>17.94</v>
-      </c>
-      <c r="F12" s="7" t="n">
-        <v>29.61</v>
       </c>
       <c r="G12" s="7">
         <f>E12-F12</f>
@@ -1564,23 +1564,23 @@
         <v/>
       </c>
       <c r="I12" s="7" t="n">
-        <v>40.25</v>
+        <v>221.53</v>
       </c>
       <c r="J12" s="6" t="n">
+        <v>2</v>
+      </c>
+      <c r="K12" s="6" t="n">
         <v>1</v>
-      </c>
-      <c r="K12" s="6" t="n">
-        <v>2</v>
       </c>
       <c r="L12" s="5">
         <f>IF(K12=0,"",(J12-K12)/K12)</f>
         <v/>
       </c>
       <c r="M12" s="6" t="n">
-        <v>5</v>
+        <v>14</v>
       </c>
       <c r="N12" s="6" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="O12" s="7">
         <f>IF(J12=0,"",E12/J12)</f>
@@ -1593,7 +1593,7 @@
         <v>454</v>
       </c>
       <c r="R12" s="7" t="n">
-        <v>10.66</v>
+        <v>31.82</v>
       </c>
       <c r="S12" s="2">
         <f>IF(AND('Engine Inputs'!E12=0,R12=0),"",IF('Engine Inputs'!E12=0,"📈 Up",IF((R12-'Engine Inputs'!E12)/'Engine Inputs'!E12&gt;Config!$B$2,"📈 Up",IF((R12-'Engine Inputs'!E12)/'Engine Inputs'!E12&lt;-Config!$B$2,"📉 Down","➡ Stable"))))</f>
@@ -1636,13 +1636,13 @@
         </is>
       </c>
       <c r="D13" s="3" t="n">
-        <v>46236</v>
+        <v>46237</v>
       </c>
       <c r="E13" s="4" t="n">
+        <v>60.16</v>
+      </c>
+      <c r="F13" s="4" t="n">
         <v>50.82</v>
-      </c>
-      <c r="F13" s="4" t="n">
-        <v>89.38</v>
       </c>
       <c r="G13" s="4">
         <f>E13-F13</f>
@@ -1653,36 +1653,36 @@
         <v/>
       </c>
       <c r="I13" s="4" t="n">
-        <v>50.4</v>
+        <v>175.02</v>
       </c>
       <c r="J13" s="6" t="n">
+        <v>7</v>
+      </c>
+      <c r="K13" s="6" t="n">
         <v>4</v>
-      </c>
-      <c r="K13" s="6" t="n">
-        <v>8</v>
       </c>
       <c r="L13" s="5">
         <f>IF(K13=0,"",(J13-K13)/K13)</f>
         <v/>
       </c>
       <c r="M13" s="6" t="n">
-        <v>5</v>
+        <v>9</v>
       </c>
       <c r="N13" s="6" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="O13" s="4">
         <f>IF(J13=0,"",E13/J13)</f>
         <v/>
       </c>
       <c r="P13" s="6" t="n">
-        <v>484</v>
+        <v>485</v>
       </c>
       <c r="Q13" s="6" t="n">
-        <v>484</v>
+        <v>485</v>
       </c>
       <c r="R13" s="4" t="n">
-        <v>52.48</v>
+        <v>60.16</v>
       </c>
       <c r="S13" s="2">
         <f>IF(AND('Engine Inputs'!E13=0,R13=0),"",IF('Engine Inputs'!E13=0,"📈 Up",IF((R13-'Engine Inputs'!E13)/'Engine Inputs'!E13&gt;Config!$B$2,"📈 Up",IF((R13-'Engine Inputs'!E13)/'Engine Inputs'!E13&lt;-Config!$B$2,"📉 Down","➡ Stable"))))</f>
@@ -1725,13 +1725,13 @@
         </is>
       </c>
       <c r="D14" s="3" t="n">
-        <v>46236</v>
+        <v>46237</v>
       </c>
       <c r="E14" s="4" t="n">
+        <v>18.47</v>
+      </c>
+      <c r="F14" s="4" t="n">
         <v>25.63</v>
-      </c>
-      <c r="F14" s="4" t="n">
-        <v>0</v>
       </c>
       <c r="G14" s="4">
         <f>E14-F14</f>
@@ -1742,23 +1742,23 @@
         <v/>
       </c>
       <c r="I14" s="4" t="n">
-        <v>45.37</v>
+        <v>74.05</v>
       </c>
       <c r="J14" s="6" t="n">
         <v>2</v>
       </c>
       <c r="K14" s="6" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="L14" s="5">
         <f>IF(K14=0,"",(J14-K14)/K14)</f>
         <v/>
       </c>
       <c r="M14" s="6" t="n">
-        <v>3</v>
+        <v>7</v>
       </c>
       <c r="N14" s="6" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="O14" s="4">
         <f>IF(J14=0,"",E14/J14)</f>
@@ -1771,7 +1771,7 @@
         <v>433</v>
       </c>
       <c r="R14" s="4" t="n">
-        <v>25.63</v>
+        <v>18.47</v>
       </c>
       <c r="S14" s="2">
         <f>IF(AND('Engine Inputs'!E14=0,R14=0),"",IF('Engine Inputs'!E14=0,"📈 Up",IF((R14-'Engine Inputs'!E14)/'Engine Inputs'!E14&gt;Config!$B$2,"📈 Up",IF((R14-'Engine Inputs'!E14)/'Engine Inputs'!E14&lt;-Config!$B$2,"📉 Down","➡ Stable"))))</f>
@@ -1814,7 +1814,7 @@
         </is>
       </c>
       <c r="D15" s="3" t="n">
-        <v>46236</v>
+        <v>46237</v>
       </c>
       <c r="E15" s="7" t="n">
         <v>0</v>
@@ -1903,7 +1903,7 @@
         </is>
       </c>
       <c r="D16" s="3" t="n">
-        <v>46236</v>
+        <v>46237</v>
       </c>
       <c r="E16" s="9" t="n">
         <v>0</v>
@@ -1992,13 +1992,13 @@
         </is>
       </c>
       <c r="D17" s="3" t="n">
-        <v>46236</v>
+        <v>46237</v>
       </c>
       <c r="E17" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="F17" s="9" t="n">
         <v>42.37</v>
-      </c>
-      <c r="F17" s="9" t="n">
-        <v>0</v>
       </c>
       <c r="G17" s="9">
         <f>E17-F17</f>
@@ -2012,10 +2012,10 @@
         <v>0</v>
       </c>
       <c r="J17" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="K17" s="6" t="n">
         <v>2</v>
-      </c>
-      <c r="K17" s="6" t="n">
-        <v>0</v>
       </c>
       <c r="L17" s="5">
         <f>IF(K17=0,"",(J17-K17)/K17)</f>
@@ -2025,7 +2025,7 @@
         <v>0</v>
       </c>
       <c r="N17" s="6" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="O17" s="9">
         <f>IF(J17=0,"",E17/J17)</f>
@@ -2038,7 +2038,7 @@
         <v>377</v>
       </c>
       <c r="R17" s="9" t="n">
-        <v>39.49</v>
+        <v>0</v>
       </c>
       <c r="S17" s="2">
         <f>IF(AND('Engine Inputs'!E17=0,R17=0),"",IF('Engine Inputs'!E17=0,"📈 Up",IF((R17-'Engine Inputs'!E17)/'Engine Inputs'!E17&gt;Config!$B$2,"📈 Up",IF((R17-'Engine Inputs'!E17)/'Engine Inputs'!E17&lt;-Config!$B$2,"📉 Down","➡ Stable"))))</f>
@@ -2081,7 +2081,7 @@
         </is>
       </c>
       <c r="D18" s="3" t="n">
-        <v>46236</v>
+        <v>46237</v>
       </c>
       <c r="E18" s="9" t="n">
         <v>0</v>
@@ -2170,13 +2170,13 @@
         </is>
       </c>
       <c r="D19" s="3" t="n">
-        <v>46236</v>
+        <v>46237</v>
       </c>
       <c r="E19" s="7" t="n">
+        <v>56.28</v>
+      </c>
+      <c r="F19" s="7" t="n">
         <v>80.16</v>
-      </c>
-      <c r="F19" s="7" t="n">
-        <v>126.54</v>
       </c>
       <c r="G19" s="7">
         <f>E19-F19</f>
@@ -2187,13 +2187,13 @@
         <v/>
       </c>
       <c r="I19" s="7" t="n">
-        <v>86.63</v>
+        <v>196.39</v>
       </c>
       <c r="J19" s="6" t="n">
+        <v>5</v>
+      </c>
+      <c r="K19" s="6" t="n">
         <v>3</v>
-      </c>
-      <c r="K19" s="6" t="n">
-        <v>4</v>
       </c>
       <c r="L19" s="5">
         <f>IF(K19=0,"",(J19-K19)/K19)</f>
@@ -2216,7 +2216,7 @@
         <v>295</v>
       </c>
       <c r="R19" s="7" t="n">
-        <v>67.37</v>
+        <v>41.9</v>
       </c>
       <c r="S19" s="2">
         <f>IF(AND('Engine Inputs'!E19=0,R19=0),"",IF('Engine Inputs'!E19=0,"📈 Up",IF((R19-'Engine Inputs'!E19)/'Engine Inputs'!E19&gt;Config!$B$2,"📈 Up",IF((R19-'Engine Inputs'!E19)/'Engine Inputs'!E19&lt;-Config!$B$2,"📉 Down","➡ Stable"))))</f>
@@ -2259,13 +2259,13 @@
         </is>
       </c>
       <c r="D20" s="3" t="n">
-        <v>46236</v>
+        <v>46237</v>
       </c>
       <c r="E20" s="4" t="n">
+        <v>21.28</v>
+      </c>
+      <c r="F20" s="4" t="n">
         <v>6.49</v>
-      </c>
-      <c r="F20" s="4" t="n">
-        <v>20.37</v>
       </c>
       <c r="G20" s="4">
         <f>E20-F20</f>
@@ -2276,10 +2276,10 @@
         <v/>
       </c>
       <c r="I20" s="4" t="n">
-        <v>56.94</v>
+        <v>26.26</v>
       </c>
       <c r="J20" s="6" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="K20" s="6" t="n">
         <v>1</v>
@@ -2292,20 +2292,20 @@
         <v>3</v>
       </c>
       <c r="N20" s="6" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="O20" s="4">
         <f>IF(J20=0,"",E20/J20)</f>
         <v/>
       </c>
       <c r="P20" s="6" t="n">
-        <v>263</v>
+        <v>264</v>
       </c>
       <c r="Q20" s="6" t="n">
-        <v>263</v>
+        <v>264</v>
       </c>
       <c r="R20" s="4" t="n">
-        <v>6.49</v>
+        <v>21.28</v>
       </c>
       <c r="S20" s="2">
         <f>IF(AND('Engine Inputs'!E20=0,R20=0),"",IF('Engine Inputs'!E20=0,"📈 Up",IF((R20-'Engine Inputs'!E20)/'Engine Inputs'!E20&gt;Config!$B$2,"📈 Up",IF((R20-'Engine Inputs'!E20)/'Engine Inputs'!E20&lt;-Config!$B$2,"📉 Down","➡ Stable"))))</f>
@@ -2334,29 +2334,29 @@
     <row r="21">
       <c r="A21" s="2" t="inlineStr">
         <is>
-          <t>LEDSone UK</t>
+          <t>Homin GmbH</t>
         </is>
       </c>
       <c r="B21" s="2" t="inlineStr">
         <is>
-          <t>Canada</t>
+          <t>Germany</t>
         </is>
       </c>
       <c r="C21" s="2" t="inlineStr">
         <is>
-          <t>CAD</t>
+          <t>EUR</t>
         </is>
       </c>
       <c r="D21" s="3" t="n">
-        <v>46236</v>
-      </c>
-      <c r="E21" s="10" t="n">
-        <v>0</v>
-      </c>
-      <c r="F21" s="10" t="n">
-        <v>0</v>
-      </c>
-      <c r="G21" s="10">
+        <v>46237</v>
+      </c>
+      <c r="E21" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="F21" s="7" t="n">
+        <v>47.98</v>
+      </c>
+      <c r="G21" s="7">
         <f>E21-F21</f>
         <v/>
       </c>
@@ -2364,14 +2364,14 @@
         <f>IF(F21=0,"",(E21-F21)/F21)</f>
         <v/>
       </c>
-      <c r="I21" s="10" t="n">
+      <c r="I21" s="7" t="n">
         <v>0</v>
       </c>
       <c r="J21" s="6" t="n">
         <v>0</v>
       </c>
       <c r="K21" s="6" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="L21" s="5">
         <f>IF(K21=0,"",(J21-K21)/K21)</f>
@@ -2383,17 +2383,17 @@
       <c r="N21" s="6" t="n">
         <v>0</v>
       </c>
-      <c r="O21" s="10">
+      <c r="O21" s="7">
         <f>IF(J21=0,"",E21/J21)</f>
         <v/>
       </c>
       <c r="P21" s="6" t="n">
-        <v>184</v>
+        <v>192</v>
       </c>
       <c r="Q21" s="6" t="n">
-        <v>184</v>
-      </c>
-      <c r="R21" s="10" t="n">
+        <v>192</v>
+      </c>
+      <c r="R21" s="7" t="n">
         <v>0</v>
       </c>
       <c r="S21" s="2">
@@ -2403,7 +2403,7 @@
       <c r="T21" s="6" t="n">
         <v>0</v>
       </c>
-      <c r="U21" s="10" t="n">
+      <c r="U21" s="7" t="n">
         <v>0</v>
       </c>
       <c r="V21" s="2">
@@ -2414,9 +2414,9 @@
         <f>IF(AND(F21=0,E21=0),"",IF(F21=0,"📈 Up",IF((E21-F21)/F21&gt;Config!$B$2,"📈 Up",IF((E21-F21)/F21&lt;-Config!$B$2,"📉 Down","➡ Stable"))))</f>
         <v/>
       </c>
-      <c r="X21" s="2" t="inlineStr">
-        <is>
-          <t>Sharmilan</t>
+      <c r="X21" s="8" t="inlineStr">
+        <is>
+          <t>— not assigned</t>
         </is>
       </c>
     </row>
@@ -2428,24 +2428,24 @@
       </c>
       <c r="B22" s="2" t="inlineStr">
         <is>
-          <t>Italy</t>
+          <t>Canada</t>
         </is>
       </c>
       <c r="C22" s="2" t="inlineStr">
         <is>
-          <t>EUR</t>
+          <t>CAD</t>
         </is>
       </c>
       <c r="D22" s="3" t="n">
-        <v>46236</v>
-      </c>
-      <c r="E22" s="7" t="n">
-        <v>102.98</v>
-      </c>
-      <c r="F22" s="7" t="n">
-        <v>0</v>
-      </c>
-      <c r="G22" s="7">
+        <v>46237</v>
+      </c>
+      <c r="E22" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="F22" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="G22" s="10">
         <f>E22-F22</f>
         <v/>
       </c>
@@ -2453,11 +2453,11 @@
         <f>IF(F22=0,"",(E22-F22)/F22)</f>
         <v/>
       </c>
-      <c r="I22" s="7" t="n">
+      <c r="I22" s="10" t="n">
         <v>0</v>
       </c>
       <c r="J22" s="6" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K22" s="6" t="n">
         <v>0</v>
@@ -2470,20 +2470,20 @@
         <v>0</v>
       </c>
       <c r="N22" s="6" t="n">
-        <v>4</v>
-      </c>
-      <c r="O22" s="7">
+        <v>0</v>
+      </c>
+      <c r="O22" s="10">
         <f>IF(J22=0,"",E22/J22)</f>
         <v/>
       </c>
       <c r="P22" s="6" t="n">
-        <v>177</v>
+        <v>184</v>
       </c>
       <c r="Q22" s="6" t="n">
-        <v>177</v>
-      </c>
-      <c r="R22" s="7" t="n">
-        <v>71.28</v>
+        <v>184</v>
+      </c>
+      <c r="R22" s="10" t="n">
+        <v>0</v>
       </c>
       <c r="S22" s="2">
         <f>IF(AND('Engine Inputs'!E22=0,R22=0),"",IF('Engine Inputs'!E22=0,"📈 Up",IF((R22-'Engine Inputs'!E22)/'Engine Inputs'!E22&gt;Config!$B$2,"📈 Up",IF((R22-'Engine Inputs'!E22)/'Engine Inputs'!E22&lt;-Config!$B$2,"📉 Down","➡ Stable"))))</f>
@@ -2492,7 +2492,7 @@
       <c r="T22" s="6" t="n">
         <v>0</v>
       </c>
-      <c r="U22" s="7" t="n">
+      <c r="U22" s="10" t="n">
         <v>0</v>
       </c>
       <c r="V22" s="2">
@@ -2512,12 +2512,12 @@
     <row r="23">
       <c r="A23" s="2" t="inlineStr">
         <is>
-          <t>Homin GmbH</t>
+          <t>LEDSone UK</t>
         </is>
       </c>
       <c r="B23" s="2" t="inlineStr">
         <is>
-          <t>Germany</t>
+          <t>Italy</t>
         </is>
       </c>
       <c r="C23" s="2" t="inlineStr">
@@ -2526,13 +2526,13 @@
         </is>
       </c>
       <c r="D23" s="3" t="n">
-        <v>46236</v>
+        <v>46237</v>
       </c>
       <c r="E23" s="7" t="n">
-        <v>47.98</v>
+        <v>0</v>
       </c>
       <c r="F23" s="7" t="n">
-        <v>10.99</v>
+        <v>102.98</v>
       </c>
       <c r="G23" s="7">
         <f>E23-F23</f>
@@ -2543,10 +2543,10 @@
         <v/>
       </c>
       <c r="I23" s="7" t="n">
-        <v>22.95</v>
+        <v>0</v>
       </c>
       <c r="J23" s="6" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="K23" s="6" t="n">
         <v>1</v>
@@ -2556,23 +2556,23 @@
         <v/>
       </c>
       <c r="M23" s="6" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="N23" s="6" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="O23" s="7">
         <f>IF(J23=0,"",E23/J23)</f>
         <v/>
       </c>
       <c r="P23" s="6" t="n">
-        <v>174</v>
+        <v>177</v>
       </c>
       <c r="Q23" s="6" t="n">
-        <v>174</v>
+        <v>177</v>
       </c>
       <c r="R23" s="7" t="n">
-        <v>47.98</v>
+        <v>0</v>
       </c>
       <c r="S23" s="2">
         <f>IF(AND('Engine Inputs'!E23=0,R23=0),"",IF('Engine Inputs'!E23=0,"📈 Up",IF((R23-'Engine Inputs'!E23)/'Engine Inputs'!E23&gt;Config!$B$2,"📈 Up",IF((R23-'Engine Inputs'!E23)/'Engine Inputs'!E23&lt;-Config!$B$2,"📉 Down","➡ Stable"))))</f>
@@ -2592,9 +2592,9 @@
         <f>IF(AND(F23=0,E23=0),"",IF(F23=0,"📈 Up",IF((E23-F23)/F23&gt;Config!$B$2,"📈 Up",IF((E23-F23)/F23&lt;-Config!$B$2,"📉 Down","➡ Stable"))))</f>
         <v/>
       </c>
-      <c r="X23" s="8" t="inlineStr">
-        <is>
-          <t>— not assigned</t>
+      <c r="X23" s="2" t="inlineStr">
+        <is>
+          <t>Sharmilan</t>
         </is>
       </c>
     </row>
@@ -2615,7 +2615,7 @@
         </is>
       </c>
       <c r="D24" s="3" t="n">
-        <v>46236</v>
+        <v>46237</v>
       </c>
       <c r="E24" s="7" t="n">
         <v>0</v>
@@ -2704,7 +2704,7 @@
         </is>
       </c>
       <c r="D25" s="3" t="n">
-        <v>46236</v>
+        <v>46237</v>
       </c>
       <c r="E25" s="10" t="n">
         <v>0</v>
@@ -2793,7 +2793,7 @@
         </is>
       </c>
       <c r="D26" s="3" t="n">
-        <v>46236</v>
+        <v>46237</v>
       </c>
       <c r="E26" s="7" t="n">
         <v>0</v>
@@ -2882,7 +2882,7 @@
         </is>
       </c>
       <c r="D27" s="3" t="n">
-        <v>46236</v>
+        <v>46237</v>
       </c>
       <c r="E27" s="4" t="n">
         <v>0</v>
@@ -2971,7 +2971,7 @@
         </is>
       </c>
       <c r="D28" s="3" t="n">
-        <v>46236</v>
+        <v>46237</v>
       </c>
       <c r="E28" s="7" t="n">
         <v>0</v>
@@ -3060,7 +3060,7 @@
         </is>
       </c>
       <c r="D29" s="3" t="n">
-        <v>46236</v>
+        <v>46237</v>
       </c>
       <c r="E29" s="7" t="n">
         <v>0</v>
@@ -3149,7 +3149,7 @@
         </is>
       </c>
       <c r="D30" s="3" t="n">
-        <v>46236</v>
+        <v>46237</v>
       </c>
       <c r="E30" s="9" t="n">
         <v>0</v>
@@ -3238,7 +3238,7 @@
         </is>
       </c>
       <c r="D31" s="3" t="n">
-        <v>46236</v>
+        <v>46237</v>
       </c>
       <c r="E31" s="7" t="n">
         <v>0</v>
@@ -3327,7 +3327,7 @@
         </is>
       </c>
       <c r="D32" s="3" t="n">
-        <v>46236</v>
+        <v>46237</v>
       </c>
       <c r="E32" s="4" t="n">
         <v>0</v>
@@ -3344,7 +3344,7 @@
         <v/>
       </c>
       <c r="I32" s="4" t="n">
-        <v>6.46</v>
+        <v>0</v>
       </c>
       <c r="J32" s="6" t="n">
         <v>0</v>
@@ -3357,7 +3357,7 @@
         <v/>
       </c>
       <c r="M32" s="6" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="N32" s="6" t="n">
         <v>0</v>
@@ -3416,7 +3416,7 @@
         </is>
       </c>
       <c r="D33" s="3" t="n">
-        <v>46236</v>
+        <v>46237</v>
       </c>
       <c r="E33" s="7" t="n">
         <v>0</v>
@@ -3521,7 +3521,7 @@
         </is>
       </c>
       <c r="B2" s="12" t="n">
-        <v>46236</v>
+        <v>46237</v>
       </c>
     </row>
     <row r="3">
@@ -3531,7 +3531,7 @@
         </is>
       </c>
       <c r="B3" s="12" t="n">
-        <v>46237</v>
+        <v>46238</v>
       </c>
     </row>
     <row r="5">
@@ -3943,12 +3943,12 @@
       </c>
       <c r="D1" s="13" t="inlineStr">
         <is>
-          <t>PH Sales 2026-08-01</t>
+          <t>PH Sales 2026-08-02</t>
         </is>
       </c>
       <c r="E1" s="13" t="inlineStr">
         <is>
-          <t>AH Sales 2026-08-01</t>
+          <t>AH Sales 2026-08-02</t>
         </is>
       </c>
       <c r="F1" s="15" t="inlineStr">
@@ -3974,10 +3974,10 @@
         </is>
       </c>
       <c r="D2" s="16" t="n">
-        <v>684.66</v>
+        <v>548.76</v>
       </c>
       <c r="E2" s="16" t="n">
-        <v>259.71</v>
+        <v>568.36</v>
       </c>
     </row>
     <row r="3">
@@ -3997,10 +3997,10 @@
         </is>
       </c>
       <c r="D3" s="16" t="n">
-        <v>296.46</v>
+        <v>147.44</v>
       </c>
       <c r="E3" s="16" t="n">
-        <v>275.49</v>
+        <v>222.27</v>
       </c>
     </row>
     <row r="4">
@@ -4020,10 +4020,10 @@
         </is>
       </c>
       <c r="D4" s="17" t="n">
-        <v>37.57</v>
+        <v>16.7</v>
       </c>
       <c r="E4" s="17" t="n">
-        <v>152.71</v>
+        <v>273.58</v>
       </c>
     </row>
     <row r="5">
@@ -4043,10 +4043,10 @@
         </is>
       </c>
       <c r="D5" s="16" t="n">
-        <v>134.89</v>
+        <v>78.81</v>
       </c>
       <c r="E5" s="16" t="n">
-        <v>142.53</v>
+        <v>206.2</v>
       </c>
     </row>
     <row r="6">
@@ -4066,10 +4066,10 @@
         </is>
       </c>
       <c r="D6" s="17" t="n">
-        <v>0</v>
+        <v>48.65</v>
       </c>
       <c r="E6" s="17" t="n">
-        <v>429.05</v>
+        <v>223.46</v>
       </c>
     </row>
     <row r="7">
@@ -4138,7 +4138,7 @@
         <v>0</v>
       </c>
       <c r="E9" s="16" t="n">
-        <v>228.49</v>
+        <v>186.65</v>
       </c>
     </row>
     <row r="10">
@@ -4158,10 +4158,10 @@
         </is>
       </c>
       <c r="D10" s="17" t="n">
-        <v>27.53</v>
+        <v>47.37</v>
       </c>
       <c r="E10" s="17" t="n">
-        <v>149.38</v>
+        <v>608.15</v>
       </c>
     </row>
     <row r="11">
@@ -4184,7 +4184,7 @@
         <v>0</v>
       </c>
       <c r="E11" s="16" t="n">
-        <v>47.48</v>
+        <v>50.29</v>
       </c>
     </row>
     <row r="12">
@@ -4207,7 +4207,7 @@
         <v>0</v>
       </c>
       <c r="E12" s="17" t="n">
-        <v>14.97</v>
+        <v>10.66</v>
       </c>
     </row>
     <row r="13">
@@ -4230,7 +4230,7 @@
         <v>0</v>
       </c>
       <c r="E13" s="16" t="n">
-        <v>87.95</v>
+        <v>52.48</v>
       </c>
     </row>
     <row r="14">
@@ -4253,7 +4253,7 @@
         <v>0</v>
       </c>
       <c r="E14" s="16" t="n">
-        <v>0</v>
+        <v>25.63</v>
       </c>
     </row>
     <row r="15">
@@ -4322,7 +4322,7 @@
         <v>0</v>
       </c>
       <c r="E17" s="18" t="n">
-        <v>0</v>
+        <v>39.49</v>
       </c>
     </row>
     <row r="18">
@@ -4368,7 +4368,7 @@
         <v>0</v>
       </c>
       <c r="E19" s="17" t="n">
-        <v>100.22</v>
+        <v>67.37</v>
       </c>
     </row>
     <row r="20">
@@ -4391,30 +4391,30 @@
         <v>0</v>
       </c>
       <c r="E20" s="16" t="n">
-        <v>20.37</v>
+        <v>6.49</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="2" t="inlineStr">
         <is>
-          <t>LEDSone UK</t>
+          <t>Homin GmbH</t>
         </is>
       </c>
       <c r="B21" s="2" t="inlineStr">
         <is>
-          <t>Canada</t>
+          <t>Germany</t>
         </is>
       </c>
       <c r="C21" s="2" t="inlineStr">
         <is>
-          <t>CAD</t>
-        </is>
-      </c>
-      <c r="D21" s="19" t="n">
-        <v>0</v>
-      </c>
-      <c r="E21" s="19" t="n">
-        <v>0</v>
+          <t>EUR</t>
+        </is>
+      </c>
+      <c r="D21" s="17" t="n">
+        <v>0</v>
+      </c>
+      <c r="E21" s="17" t="n">
+        <v>47.98</v>
       </c>
     </row>
     <row r="22">
@@ -4425,30 +4425,30 @@
       </c>
       <c r="B22" s="2" t="inlineStr">
         <is>
-          <t>Italy</t>
+          <t>Canada</t>
         </is>
       </c>
       <c r="C22" s="2" t="inlineStr">
         <is>
-          <t>EUR</t>
-        </is>
-      </c>
-      <c r="D22" s="17" t="n">
-        <v>0</v>
-      </c>
-      <c r="E22" s="17" t="n">
+          <t>CAD</t>
+        </is>
+      </c>
+      <c r="D22" s="19" t="n">
+        <v>0</v>
+      </c>
+      <c r="E22" s="19" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="2" t="inlineStr">
         <is>
-          <t>Homin GmbH</t>
+          <t>LEDSone UK</t>
         </is>
       </c>
       <c r="B23" s="2" t="inlineStr">
         <is>
-          <t>Germany</t>
+          <t>Italy</t>
         </is>
       </c>
       <c r="C23" s="2" t="inlineStr">
@@ -4460,7 +4460,7 @@
         <v>0</v>
       </c>
       <c r="E23" s="17" t="n">
-        <v>10.99</v>
+        <v>71.28</v>
       </c>
     </row>
     <row r="24">
@@ -4806,7 +4806,7 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t xml:space="preserve">  Generated 2026-08-03.  "Today" = 2026-08-02.  "Yesterday" = 2026-08-01.  Same Day LY = 2025-08-02.</t>
+          <t xml:space="preserve">  Generated 2026-08-04.  "Today" = 2026-08-03.  "Yesterday" = 2026-08-02.  Same Day LY = 2025-08-03.</t>
         </is>
       </c>
     </row>
@@ -4851,7 +4851,7 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t xml:space="preserve">  Why not 'Completed' only: orders reach Completed about 2 days after purchase. On 2026-08-02</t>
+          <t xml:space="preserve">  Why not 'Completed' only: orders reach Completed about 2 days after purchase. On 2026-08-03</t>
         </is>
       </c>
     </row>
@@ -5162,7 +5162,7 @@
     <row r="72">
       <c r="A72" t="inlineStr">
         <is>
-          <t xml:space="preserve">  (2026-08-02 was a Sunday; 2025-08-02 was a Saturday). Day-of-week effects are present in this comparison.</t>
+          <t xml:space="preserve">  (2026-08-03 was a Monday; 2025-08-03 was a Sunday). Day-of-week effects are present in this comparison.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
chore(aios): commit uncommitted report outputs and review documents
Housekeeping only, no code or automation changes. EPPA/DST/Meshika report outputs regenerated by their own jobs, 3 docx briefs, 2 review notes, 2 CHOP payload snapshots. Screened: 3.2 MB, no credentials or DB hosts in any text file.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/development/abiraj_mini_aios_workbench/projects/PRJ-2026-015_daily-sales-track/evidence/final_outputs/REQ-17_daily-sales-track/REQ-17-D01_daily_sales_track.xlsx
+++ b/development/abiraj_mini_aios_workbench/projects/PRJ-2026-015_daily-sales-track/evidence/final_outputs/REQ-17_daily-sales-track/REQ-17-D01_daily_sales_track.xlsx
@@ -657,13 +657,13 @@
         </is>
       </c>
       <c r="D2" s="3" t="n">
-        <v>46247</v>
+        <v>46251</v>
       </c>
       <c r="E2" s="4" t="n">
-        <v>965.86</v>
+        <v>1122.21</v>
       </c>
       <c r="F2" s="4" t="n">
-        <v>816.55</v>
+        <v>1160.45</v>
       </c>
       <c r="G2" s="4">
         <f>E2-F2</f>
@@ -674,36 +674,36 @@
         <v/>
       </c>
       <c r="I2" s="4" t="n">
-        <v>1219.5</v>
+        <v>928.1</v>
       </c>
       <c r="J2" s="6" t="n">
-        <v>53</v>
+        <v>67</v>
       </c>
       <c r="K2" s="6" t="n">
-        <v>47</v>
+        <v>65</v>
       </c>
       <c r="L2" s="5">
         <f>IF(K2=0,"",(J2-K2)/K2)</f>
         <v/>
       </c>
       <c r="M2" s="6" t="n">
-        <v>72</v>
+        <v>69</v>
       </c>
       <c r="N2" s="6" t="n">
-        <v>98</v>
+        <v>104</v>
       </c>
       <c r="O2" s="4">
         <f>IF(J2=0,"",E2/J2)</f>
         <v/>
       </c>
       <c r="P2" s="6" t="n">
-        <v>3058</v>
+        <v>3062</v>
       </c>
       <c r="Q2" s="6" t="n">
-        <v>1752</v>
+        <v>1756</v>
       </c>
       <c r="R2" s="4" t="n">
-        <v>578.83</v>
+        <v>603.2</v>
       </c>
       <c r="S2" s="2">
         <f>IF(AND('Engine Inputs'!E2=0,R2=0),"",IF('Engine Inputs'!E2=0,"📈 Up",IF((R2-'Engine Inputs'!E2)/'Engine Inputs'!E2&gt;Config!$B$2,"📈 Up",IF((R2-'Engine Inputs'!E2)/'Engine Inputs'!E2&lt;-Config!$B$2,"📉 Down","➡ Stable"))))</f>
@@ -713,7 +713,7 @@
         <v>1306</v>
       </c>
       <c r="U2" s="4" t="n">
-        <v>379.8</v>
+        <v>517.77</v>
       </c>
       <c r="V2" s="2">
         <f>IF(AND('Engine Inputs'!D2=0,U2=0),"",IF('Engine Inputs'!D2=0,"📈 Up",IF((U2-'Engine Inputs'!D2)/'Engine Inputs'!D2&gt;Config!$B$2,"📈 Up",IF((U2-'Engine Inputs'!D2)/'Engine Inputs'!D2&lt;-Config!$B$2,"📉 Down","➡ Stable"))))</f>
@@ -746,13 +746,13 @@
         </is>
       </c>
       <c r="D3" s="3" t="n">
-        <v>46247</v>
+        <v>46251</v>
       </c>
       <c r="E3" s="4" t="n">
-        <v>299.98</v>
+        <v>537.51</v>
       </c>
       <c r="F3" s="4" t="n">
-        <v>227.41</v>
+        <v>293.97</v>
       </c>
       <c r="G3" s="4">
         <f>E3-F3</f>
@@ -763,36 +763,36 @@
         <v/>
       </c>
       <c r="I3" s="4" t="n">
-        <v>476.63</v>
+        <v>764.91</v>
       </c>
       <c r="J3" s="6" t="n">
-        <v>18</v>
+        <v>33</v>
       </c>
       <c r="K3" s="6" t="n">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="L3" s="5">
         <f>IF(K3=0,"",(J3-K3)/K3)</f>
         <v/>
       </c>
       <c r="M3" s="6" t="n">
-        <v>29</v>
+        <v>47</v>
       </c>
       <c r="N3" s="6" t="n">
-        <v>28</v>
+        <v>44</v>
       </c>
       <c r="O3" s="4">
         <f>IF(J3=0,"",E3/J3)</f>
         <v/>
       </c>
       <c r="P3" s="6" t="n">
-        <v>1695</v>
+        <v>1699</v>
       </c>
       <c r="Q3" s="6" t="n">
-        <v>1098</v>
+        <v>1102</v>
       </c>
       <c r="R3" s="4" t="n">
-        <v>42.56</v>
+        <v>306.32</v>
       </c>
       <c r="S3" s="2">
         <f>IF(AND('Engine Inputs'!E3=0,R3=0),"",IF('Engine Inputs'!E3=0,"📈 Up",IF((R3-'Engine Inputs'!E3)/'Engine Inputs'!E3&gt;Config!$B$2,"📈 Up",IF((R3-'Engine Inputs'!E3)/'Engine Inputs'!E3&lt;-Config!$B$2,"📉 Down","➡ Stable"))))</f>
@@ -802,7 +802,7 @@
         <v>597</v>
       </c>
       <c r="U3" s="4" t="n">
-        <v>261.78</v>
+        <v>237.96</v>
       </c>
       <c r="V3" s="2">
         <f>IF(AND('Engine Inputs'!D3=0,U3=0),"",IF('Engine Inputs'!D3=0,"📈 Up",IF((U3-'Engine Inputs'!D3)/'Engine Inputs'!D3&gt;Config!$B$2,"📈 Up",IF((U3-'Engine Inputs'!D3)/'Engine Inputs'!D3&lt;-Config!$B$2,"📉 Down","➡ Stable"))))</f>
@@ -835,13 +835,13 @@
         </is>
       </c>
       <c r="D4" s="3" t="n">
-        <v>46247</v>
+        <v>46251</v>
       </c>
       <c r="E4" s="7" t="n">
-        <v>252.71</v>
+        <v>302.99</v>
       </c>
       <c r="F4" s="7" t="n">
-        <v>321.17</v>
+        <v>320.86</v>
       </c>
       <c r="G4" s="7">
         <f>E4-F4</f>
@@ -852,36 +852,36 @@
         <v/>
       </c>
       <c r="I4" s="7" t="n">
-        <v>493.49</v>
+        <v>767.77</v>
       </c>
       <c r="J4" s="6" t="n">
-        <v>10</v>
+        <v>13</v>
       </c>
       <c r="K4" s="6" t="n">
-        <v>8</v>
+        <v>12</v>
       </c>
       <c r="L4" s="5">
         <f>IF(K4=0,"",(J4-K4)/K4)</f>
         <v/>
       </c>
       <c r="M4" s="6" t="n">
-        <v>17</v>
+        <v>25</v>
       </c>
       <c r="N4" s="6" t="n">
-        <v>14</v>
+        <v>16</v>
       </c>
       <c r="O4" s="7">
         <f>IF(J4=0,"",E4/J4)</f>
         <v/>
       </c>
       <c r="P4" s="6" t="n">
-        <v>1452</v>
+        <v>1453</v>
       </c>
       <c r="Q4" s="6" t="n">
-        <v>1220</v>
+        <v>1221</v>
       </c>
       <c r="R4" s="7" t="n">
-        <v>161.6</v>
+        <v>199.69</v>
       </c>
       <c r="S4" s="2">
         <f>IF(AND('Engine Inputs'!E4=0,R4=0),"",IF('Engine Inputs'!E4=0,"📈 Up",IF((R4-'Engine Inputs'!E4)/'Engine Inputs'!E4&gt;Config!$B$2,"📈 Up",IF((R4-'Engine Inputs'!E4)/'Engine Inputs'!E4&lt;-Config!$B$2,"📉 Down","➡ Stable"))))</f>
@@ -891,7 +891,7 @@
         <v>232</v>
       </c>
       <c r="U4" s="7" t="n">
-        <v>13.17</v>
+        <v>3.78</v>
       </c>
       <c r="V4" s="2">
         <f>IF(AND('Engine Inputs'!D4=0,U4=0),"",IF('Engine Inputs'!D4=0,"📈 Up",IF((U4-'Engine Inputs'!D4)/'Engine Inputs'!D4&gt;Config!$B$2,"📈 Up",IF((U4-'Engine Inputs'!D4)/'Engine Inputs'!D4&lt;-Config!$B$2,"📉 Down","➡ Stable"))))</f>
@@ -924,13 +924,13 @@
         </is>
       </c>
       <c r="D5" s="3" t="n">
-        <v>46247</v>
+        <v>46251</v>
       </c>
       <c r="E5" s="4" t="n">
-        <v>213.89</v>
+        <v>320.64</v>
       </c>
       <c r="F5" s="4" t="n">
-        <v>162.69</v>
+        <v>234.77</v>
       </c>
       <c r="G5" s="4">
         <f>E5-F5</f>
@@ -941,36 +941,36 @@
         <v/>
       </c>
       <c r="I5" s="4" t="n">
-        <v>219.38</v>
+        <v>203.52</v>
       </c>
       <c r="J5" s="6" t="n">
+        <v>18</v>
+      </c>
+      <c r="K5" s="6" t="n">
         <v>15</v>
-      </c>
-      <c r="K5" s="6" t="n">
-        <v>13</v>
       </c>
       <c r="L5" s="5">
         <f>IF(K5=0,"",(J5-K5)/K5)</f>
         <v/>
       </c>
       <c r="M5" s="6" t="n">
-        <v>17</v>
+        <v>14</v>
       </c>
       <c r="N5" s="6" t="n">
-        <v>26</v>
+        <v>34</v>
       </c>
       <c r="O5" s="4">
         <f>IF(J5=0,"",E5/J5)</f>
         <v/>
       </c>
       <c r="P5" s="6" t="n">
-        <v>1211</v>
+        <v>1214</v>
       </c>
       <c r="Q5" s="6" t="n">
-        <v>741</v>
+        <v>744</v>
       </c>
       <c r="R5" s="4" t="n">
-        <v>158.62</v>
+        <v>234.1</v>
       </c>
       <c r="S5" s="2">
         <f>IF(AND('Engine Inputs'!E5=0,R5=0),"",IF('Engine Inputs'!E5=0,"📈 Up",IF((R5-'Engine Inputs'!E5)/'Engine Inputs'!E5&gt;Config!$B$2,"📈 Up",IF((R5-'Engine Inputs'!E5)/'Engine Inputs'!E5&lt;-Config!$B$2,"📉 Down","➡ Stable"))))</f>
@@ -980,7 +980,7 @@
         <v>470</v>
       </c>
       <c r="U5" s="4" t="n">
-        <v>47.53</v>
+        <v>87.39</v>
       </c>
       <c r="V5" s="2">
         <f>IF(AND('Engine Inputs'!D5=0,U5=0),"",IF('Engine Inputs'!D5=0,"📈 Up",IF((U5-'Engine Inputs'!D5)/'Engine Inputs'!D5&gt;Config!$B$2,"📈 Up",IF((U5-'Engine Inputs'!D5)/'Engine Inputs'!D5&lt;-Config!$B$2,"📉 Down","➡ Stable"))))</f>
@@ -1013,13 +1013,13 @@
         </is>
       </c>
       <c r="D6" s="3" t="n">
-        <v>46247</v>
+        <v>46251</v>
       </c>
       <c r="E6" s="7" t="n">
-        <v>203.58</v>
+        <v>170.81</v>
       </c>
       <c r="F6" s="7" t="n">
-        <v>178.12</v>
+        <v>211.06</v>
       </c>
       <c r="G6" s="7">
         <f>E6-F6</f>
@@ -1030,36 +1030,36 @@
         <v/>
       </c>
       <c r="I6" s="7" t="n">
-        <v>317.26</v>
+        <v>337.65</v>
       </c>
       <c r="J6" s="6" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="K6" s="6" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="L6" s="5">
         <f>IF(K6=0,"",(J6-K6)/K6)</f>
         <v/>
       </c>
       <c r="M6" s="6" t="n">
-        <v>17</v>
+        <v>19</v>
       </c>
       <c r="N6" s="6" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="O6" s="7">
         <f>IF(J6=0,"",E6/J6)</f>
         <v/>
       </c>
       <c r="P6" s="6" t="n">
-        <v>669</v>
+        <v>670</v>
       </c>
       <c r="Q6" s="6" t="n">
-        <v>580</v>
+        <v>581</v>
       </c>
       <c r="R6" s="7" t="n">
-        <v>187.69</v>
+        <v>128.94</v>
       </c>
       <c r="S6" s="2">
         <f>IF(AND('Engine Inputs'!E6=0,R6=0),"",IF('Engine Inputs'!E6=0,"📈 Up",IF((R6-'Engine Inputs'!E6)/'Engine Inputs'!E6&gt;Config!$B$2,"📈 Up",IF((R6-'Engine Inputs'!E6)/'Engine Inputs'!E6&lt;-Config!$B$2,"📉 Down","➡ Stable"))))</f>
@@ -1069,7 +1069,7 @@
         <v>89</v>
       </c>
       <c r="U6" s="7" t="n">
-        <v>0</v>
+        <v>14.99</v>
       </c>
       <c r="V6" s="2">
         <f>IF(AND('Engine Inputs'!D6=0,U6=0),"",IF('Engine Inputs'!D6=0,"📈 Up",IF((U6-'Engine Inputs'!D6)/'Engine Inputs'!D6&gt;Config!$B$2,"📈 Up",IF((U6-'Engine Inputs'!D6)/'Engine Inputs'!D6&lt;-Config!$B$2,"📉 Down","➡ Stable"))))</f>
@@ -1102,7 +1102,7 @@
         </is>
       </c>
       <c r="D7" s="3" t="n">
-        <v>46247</v>
+        <v>46251</v>
       </c>
       <c r="E7" s="7" t="n">
         <v>0</v>
@@ -1191,7 +1191,7 @@
         </is>
       </c>
       <c r="D8" s="3" t="n">
-        <v>46247</v>
+        <v>46251</v>
       </c>
       <c r="E8" s="7" t="n">
         <v>0</v>
@@ -1280,13 +1280,13 @@
         </is>
       </c>
       <c r="D9" s="3" t="n">
-        <v>46247</v>
+        <v>46251</v>
       </c>
       <c r="E9" s="4" t="n">
-        <v>208.8</v>
+        <v>223.61</v>
       </c>
       <c r="F9" s="4" t="n">
-        <v>315.7</v>
+        <v>164.5</v>
       </c>
       <c r="G9" s="4">
         <f>E9-F9</f>
@@ -1297,23 +1297,23 @@
         <v/>
       </c>
       <c r="I9" s="4" t="n">
-        <v>28.02</v>
+        <v>162.52</v>
       </c>
       <c r="J9" s="6" t="n">
-        <v>12</v>
+        <v>16</v>
       </c>
       <c r="K9" s="6" t="n">
-        <v>10</v>
+        <v>7</v>
       </c>
       <c r="L9" s="5">
         <f>IF(K9=0,"",(J9-K9)/K9)</f>
         <v/>
       </c>
       <c r="M9" s="6" t="n">
-        <v>4</v>
+        <v>15</v>
       </c>
       <c r="N9" s="6" t="n">
-        <v>22</v>
+        <v>19</v>
       </c>
       <c r="O9" s="4">
         <f>IF(J9=0,"",E9/J9)</f>
@@ -1326,7 +1326,7 @@
         <v>579</v>
       </c>
       <c r="R9" s="4" t="n">
-        <v>208.8</v>
+        <v>223.61</v>
       </c>
       <c r="S9" s="2">
         <f>IF(AND('Engine Inputs'!E9=0,R9=0),"",IF('Engine Inputs'!E9=0,"📈 Up",IF((R9-'Engine Inputs'!E9)/'Engine Inputs'!E9&gt;Config!$B$2,"📈 Up",IF((R9-'Engine Inputs'!E9)/'Engine Inputs'!E9&lt;-Config!$B$2,"📉 Down","➡ Stable"))))</f>
@@ -1369,13 +1369,13 @@
         </is>
       </c>
       <c r="D10" s="3" t="n">
-        <v>46247</v>
+        <v>46251</v>
       </c>
       <c r="E10" s="7" t="n">
-        <v>326.92</v>
+        <v>288.24</v>
       </c>
       <c r="F10" s="7" t="n">
-        <v>468.51</v>
+        <v>323.05</v>
       </c>
       <c r="G10" s="7">
         <f>E10-F10</f>
@@ -1386,10 +1386,10 @@
         <v/>
       </c>
       <c r="I10" s="7" t="n">
-        <v>205.97</v>
+        <v>240.18</v>
       </c>
       <c r="J10" s="6" t="n">
-        <v>17</v>
+        <v>11</v>
       </c>
       <c r="K10" s="6" t="n">
         <v>13</v>
@@ -1399,23 +1399,23 @@
         <v/>
       </c>
       <c r="M10" s="6" t="n">
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="N10" s="6" t="n">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="O10" s="7">
         <f>IF(J10=0,"",E10/J10)</f>
         <v/>
       </c>
       <c r="P10" s="6" t="n">
-        <v>558</v>
+        <v>560</v>
       </c>
       <c r="Q10" s="6" t="n">
-        <v>465</v>
+        <v>467</v>
       </c>
       <c r="R10" s="7" t="n">
-        <v>180.33</v>
+        <v>207.36</v>
       </c>
       <c r="S10" s="2">
         <f>IF(AND('Engine Inputs'!E10=0,R10=0),"",IF('Engine Inputs'!E10=0,"📈 Up",IF((R10-'Engine Inputs'!E10)/'Engine Inputs'!E10&gt;Config!$B$2,"📈 Up",IF((R10-'Engine Inputs'!E10)/'Engine Inputs'!E10&lt;-Config!$B$2,"📉 Down","➡ Stable"))))</f>
@@ -1425,7 +1425,7 @@
         <v>93</v>
       </c>
       <c r="U10" s="7" t="n">
-        <v>62.09</v>
+        <v>37.27</v>
       </c>
       <c r="V10" s="2">
         <f>IF(AND('Engine Inputs'!D10=0,U10=0),"",IF('Engine Inputs'!D10=0,"📈 Up",IF((U10-'Engine Inputs'!D10)/'Engine Inputs'!D10&gt;Config!$B$2,"📈 Up",IF((U10-'Engine Inputs'!D10)/'Engine Inputs'!D10&lt;-Config!$B$2,"📉 Down","➡ Stable"))))</f>
@@ -1458,13 +1458,13 @@
         </is>
       </c>
       <c r="D11" s="3" t="n">
-        <v>46247</v>
+        <v>46251</v>
       </c>
       <c r="E11" s="4" t="n">
-        <v>80.05</v>
+        <v>111.89</v>
       </c>
       <c r="F11" s="4" t="n">
-        <v>36.06</v>
+        <v>78.98999999999999</v>
       </c>
       <c r="G11" s="4">
         <f>E11-F11</f>
@@ -1475,23 +1475,23 @@
         <v/>
       </c>
       <c r="I11" s="4" t="n">
-        <v>69.38</v>
+        <v>106.52</v>
       </c>
       <c r="J11" s="6" t="n">
         <v>8</v>
       </c>
       <c r="K11" s="6" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="L11" s="5">
         <f>IF(K11=0,"",(J11-K11)/K11)</f>
         <v/>
       </c>
       <c r="M11" s="6" t="n">
-        <v>8</v>
+        <v>15</v>
       </c>
       <c r="N11" s="6" t="n">
-        <v>17</v>
+        <v>14</v>
       </c>
       <c r="O11" s="4">
         <f>IF(J11=0,"",E11/J11)</f>
@@ -1504,7 +1504,7 @@
         <v>509</v>
       </c>
       <c r="R11" s="4" t="n">
-        <v>81.56999999999999</v>
+        <v>115.44</v>
       </c>
       <c r="S11" s="2">
         <f>IF(AND('Engine Inputs'!E11=0,R11=0),"",IF('Engine Inputs'!E11=0,"📈 Up",IF((R11-'Engine Inputs'!E11)/'Engine Inputs'!E11&gt;Config!$B$2,"📈 Up",IF((R11-'Engine Inputs'!E11)/'Engine Inputs'!E11&lt;-Config!$B$2,"📉 Down","➡ Stable"))))</f>
@@ -1547,13 +1547,13 @@
         </is>
       </c>
       <c r="D12" s="3" t="n">
-        <v>46247</v>
+        <v>46251</v>
       </c>
       <c r="E12" s="7" t="n">
-        <v>96.73</v>
+        <v>14.14</v>
       </c>
       <c r="F12" s="7" t="n">
-        <v>93.66</v>
+        <v>60.28</v>
       </c>
       <c r="G12" s="7">
         <f>E12-F12</f>
@@ -1564,10 +1564,10 @@
         <v/>
       </c>
       <c r="I12" s="7" t="n">
-        <v>122.78</v>
+        <v>208.28</v>
       </c>
       <c r="J12" s="6" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="K12" s="6" t="n">
         <v>4</v>
@@ -1577,10 +1577,10 @@
         <v/>
       </c>
       <c r="M12" s="6" t="n">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="N12" s="6" t="n">
-        <v>7</v>
+        <v>1</v>
       </c>
       <c r="O12" s="7">
         <f>IF(J12=0,"",E12/J12)</f>
@@ -1593,7 +1593,7 @@
         <v>454</v>
       </c>
       <c r="R12" s="7" t="n">
-        <v>64.23</v>
+        <v>7.47</v>
       </c>
       <c r="S12" s="2">
         <f>IF(AND('Engine Inputs'!E12=0,R12=0),"",IF('Engine Inputs'!E12=0,"📈 Up",IF((R12-'Engine Inputs'!E12)/'Engine Inputs'!E12&gt;Config!$B$2,"📈 Up",IF((R12-'Engine Inputs'!E12)/'Engine Inputs'!E12&lt;-Config!$B$2,"📉 Down","➡ Stable"))))</f>
@@ -1603,7 +1603,7 @@
         <v>37</v>
       </c>
       <c r="U12" s="7" t="n">
-        <v>2.85</v>
+        <v>0</v>
       </c>
       <c r="V12" s="2">
         <f>IF(AND('Engine Inputs'!D12=0,U12=0),"",IF('Engine Inputs'!D12=0,"📈 Up",IF((U12-'Engine Inputs'!D12)/'Engine Inputs'!D12&gt;Config!$B$2,"📈 Up",IF((U12-'Engine Inputs'!D12)/'Engine Inputs'!D12&lt;-Config!$B$2,"📉 Down","➡ Stable"))))</f>
@@ -1636,13 +1636,13 @@
         </is>
       </c>
       <c r="D13" s="3" t="n">
-        <v>46247</v>
+        <v>46251</v>
       </c>
       <c r="E13" s="4" t="n">
-        <v>23.91</v>
+        <v>6.99</v>
       </c>
       <c r="F13" s="4" t="n">
-        <v>109.12</v>
+        <v>102.12</v>
       </c>
       <c r="G13" s="4">
         <f>E13-F13</f>
@@ -1653,23 +1653,23 @@
         <v/>
       </c>
       <c r="I13" s="4" t="n">
-        <v>142.56</v>
+        <v>78.14</v>
       </c>
       <c r="J13" s="6" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="K13" s="6" t="n">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="L13" s="5">
         <f>IF(K13=0,"",(J13-K13)/K13)</f>
         <v/>
       </c>
       <c r="M13" s="6" t="n">
-        <v>10</v>
+        <v>7</v>
       </c>
       <c r="N13" s="6" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="O13" s="4">
         <f>IF(J13=0,"",E13/J13)</f>
@@ -1682,7 +1682,7 @@
         <v>487</v>
       </c>
       <c r="R13" s="4" t="n">
-        <v>23.91</v>
+        <v>6.99</v>
       </c>
       <c r="S13" s="2">
         <f>IF(AND('Engine Inputs'!E13=0,R13=0),"",IF('Engine Inputs'!E13=0,"📈 Up",IF((R13-'Engine Inputs'!E13)/'Engine Inputs'!E13&gt;Config!$B$2,"📈 Up",IF((R13-'Engine Inputs'!E13)/'Engine Inputs'!E13&lt;-Config!$B$2,"📉 Down","➡ Stable"))))</f>
@@ -1725,13 +1725,13 @@
         </is>
       </c>
       <c r="D14" s="3" t="n">
-        <v>46247</v>
+        <v>46251</v>
       </c>
       <c r="E14" s="4" t="n">
-        <v>0</v>
+        <v>90.76000000000001</v>
       </c>
       <c r="F14" s="4" t="n">
-        <v>65.38</v>
+        <v>14.7</v>
       </c>
       <c r="G14" s="4">
         <f>E14-F14</f>
@@ -1742,36 +1742,36 @@
         <v/>
       </c>
       <c r="I14" s="4" t="n">
-        <v>31.95</v>
+        <v>32.4</v>
       </c>
       <c r="J14" s="6" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="K14" s="6" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="L14" s="5">
         <f>IF(K14=0,"",(J14-K14)/K14)</f>
         <v/>
       </c>
       <c r="M14" s="6" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="N14" s="6" t="n">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="O14" s="4">
         <f>IF(J14=0,"",E14/J14)</f>
         <v/>
       </c>
       <c r="P14" s="6" t="n">
-        <v>434</v>
+        <v>435</v>
       </c>
       <c r="Q14" s="6" t="n">
-        <v>434</v>
+        <v>435</v>
       </c>
       <c r="R14" s="4" t="n">
-        <v>0</v>
+        <v>90.76000000000001</v>
       </c>
       <c r="S14" s="2">
         <f>IF(AND('Engine Inputs'!E14=0,R14=0),"",IF('Engine Inputs'!E14=0,"📈 Up",IF((R14-'Engine Inputs'!E14)/'Engine Inputs'!E14&gt;Config!$B$2,"📈 Up",IF((R14-'Engine Inputs'!E14)/'Engine Inputs'!E14&lt;-Config!$B$2,"📉 Down","➡ Stable"))))</f>
@@ -1814,13 +1814,13 @@
         </is>
       </c>
       <c r="D15" s="3" t="n">
-        <v>46247</v>
+        <v>46251</v>
       </c>
       <c r="E15" s="7" t="n">
         <v>0</v>
       </c>
       <c r="F15" s="7" t="n">
-        <v>0</v>
+        <v>26.73</v>
       </c>
       <c r="G15" s="7">
         <f>E15-F15</f>
@@ -1837,7 +1837,7 @@
         <v>0</v>
       </c>
       <c r="K15" s="6" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L15" s="5">
         <f>IF(K15=0,"",(J15-K15)/K15)</f>
@@ -1903,13 +1903,13 @@
         </is>
       </c>
       <c r="D16" s="3" t="n">
-        <v>46247</v>
+        <v>46251</v>
       </c>
       <c r="E16" s="9" t="n">
         <v>0</v>
       </c>
       <c r="F16" s="9" t="n">
-        <v>19.18</v>
+        <v>0</v>
       </c>
       <c r="G16" s="9">
         <f>E16-F16</f>
@@ -1920,20 +1920,20 @@
         <v/>
       </c>
       <c r="I16" s="9" t="n">
-        <v>36.25</v>
+        <v>0</v>
       </c>
       <c r="J16" s="6" t="n">
         <v>0</v>
       </c>
       <c r="K16" s="6" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="L16" s="5">
         <f>IF(K16=0,"",(J16-K16)/K16)</f>
         <v/>
       </c>
       <c r="M16" s="6" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="N16" s="6" t="n">
         <v>0</v>
@@ -1992,13 +1992,13 @@
         </is>
       </c>
       <c r="D17" s="3" t="n">
-        <v>46247</v>
+        <v>46251</v>
       </c>
       <c r="E17" s="9" t="n">
-        <v>0</v>
+        <v>28.47</v>
       </c>
       <c r="F17" s="9" t="n">
-        <v>0</v>
+        <v>15.19</v>
       </c>
       <c r="G17" s="9">
         <f>E17-F17</f>
@@ -2012,10 +2012,10 @@
         <v>0</v>
       </c>
       <c r="J17" s="6" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K17" s="6" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L17" s="5">
         <f>IF(K17=0,"",(J17-K17)/K17)</f>
@@ -2025,7 +2025,7 @@
         <v>0</v>
       </c>
       <c r="N17" s="6" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="O17" s="9">
         <f>IF(J17=0,"",E17/J17)</f>
@@ -2038,7 +2038,7 @@
         <v>377</v>
       </c>
       <c r="R17" s="9" t="n">
-        <v>0</v>
+        <v>26.99</v>
       </c>
       <c r="S17" s="2">
         <f>IF(AND('Engine Inputs'!E17=0,R17=0),"",IF('Engine Inputs'!E17=0,"📈 Up",IF((R17-'Engine Inputs'!E17)/'Engine Inputs'!E17&gt;Config!$B$2,"📈 Up",IF((R17-'Engine Inputs'!E17)/'Engine Inputs'!E17&lt;-Config!$B$2,"📉 Down","➡ Stable"))))</f>
@@ -2081,13 +2081,13 @@
         </is>
       </c>
       <c r="D18" s="3" t="n">
-        <v>46247</v>
+        <v>46251</v>
       </c>
       <c r="E18" s="9" t="n">
-        <v>0</v>
+        <v>23.44</v>
       </c>
       <c r="F18" s="9" t="n">
-        <v>0</v>
+        <v>145.04</v>
       </c>
       <c r="G18" s="9">
         <f>E18-F18</f>
@@ -2101,10 +2101,10 @@
         <v>0</v>
       </c>
       <c r="J18" s="6" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K18" s="6" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="L18" s="5">
         <f>IF(K18=0,"",(J18-K18)/K18)</f>
@@ -2114,7 +2114,7 @@
         <v>0</v>
       </c>
       <c r="N18" s="6" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="O18" s="9">
         <f>IF(J18=0,"",E18/J18)</f>
@@ -2127,7 +2127,7 @@
         <v>329</v>
       </c>
       <c r="R18" s="9" t="n">
-        <v>0</v>
+        <v>21.5</v>
       </c>
       <c r="S18" s="2">
         <f>IF(AND('Engine Inputs'!E18=0,R18=0),"",IF('Engine Inputs'!E18=0,"📈 Up",IF((R18-'Engine Inputs'!E18)/'Engine Inputs'!E18&gt;Config!$B$2,"📈 Up",IF((R18-'Engine Inputs'!E18)/'Engine Inputs'!E18&lt;-Config!$B$2,"📉 Down","➡ Stable"))))</f>
@@ -2170,10 +2170,10 @@
         </is>
       </c>
       <c r="D19" s="3" t="n">
-        <v>46247</v>
+        <v>46251</v>
       </c>
       <c r="E19" s="7" t="n">
-        <v>33.25</v>
+        <v>0</v>
       </c>
       <c r="F19" s="7" t="n">
         <v>0</v>
@@ -2187,10 +2187,10 @@
         <v/>
       </c>
       <c r="I19" s="7" t="n">
-        <v>37.19</v>
+        <v>117.93</v>
       </c>
       <c r="J19" s="6" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="K19" s="6" t="n">
         <v>0</v>
@@ -2203,20 +2203,20 @@
         <v>6</v>
       </c>
       <c r="N19" s="6" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="O19" s="7">
         <f>IF(J19=0,"",E19/J19)</f>
         <v/>
       </c>
       <c r="P19" s="6" t="n">
-        <v>300</v>
+        <v>301</v>
       </c>
       <c r="Q19" s="6" t="n">
-        <v>300</v>
+        <v>301</v>
       </c>
       <c r="R19" s="7" t="n">
-        <v>19.12</v>
+        <v>0</v>
       </c>
       <c r="S19" s="2">
         <f>IF(AND('Engine Inputs'!E19=0,R19=0),"",IF('Engine Inputs'!E19=0,"📈 Up",IF((R19-'Engine Inputs'!E19)/'Engine Inputs'!E19&gt;Config!$B$2,"📈 Up",IF((R19-'Engine Inputs'!E19)/'Engine Inputs'!E19&lt;-Config!$B$2,"📉 Down","➡ Stable"))))</f>
@@ -2259,13 +2259,13 @@
         </is>
       </c>
       <c r="D20" s="3" t="n">
-        <v>46247</v>
+        <v>46251</v>
       </c>
       <c r="E20" s="4" t="n">
-        <v>5.89</v>
+        <v>34.88</v>
       </c>
       <c r="F20" s="4" t="n">
-        <v>10.78</v>
+        <v>0</v>
       </c>
       <c r="G20" s="4">
         <f>E20-F20</f>
@@ -2276,36 +2276,36 @@
         <v/>
       </c>
       <c r="I20" s="4" t="n">
-        <v>14.89</v>
+        <v>71.70999999999999</v>
       </c>
       <c r="J20" s="6" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="K20" s="6" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="L20" s="5">
         <f>IF(K20=0,"",(J20-K20)/K20)</f>
         <v/>
       </c>
       <c r="M20" s="6" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="N20" s="6" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="O20" s="4">
         <f>IF(J20=0,"",E20/J20)</f>
         <v/>
       </c>
       <c r="P20" s="6" t="n">
-        <v>265</v>
+        <v>266</v>
       </c>
       <c r="Q20" s="6" t="n">
-        <v>265</v>
+        <v>266</v>
       </c>
       <c r="R20" s="4" t="n">
-        <v>5.89</v>
+        <v>34.88</v>
       </c>
       <c r="S20" s="2">
         <f>IF(AND('Engine Inputs'!E20=0,R20=0),"",IF('Engine Inputs'!E20=0,"📈 Up",IF((R20-'Engine Inputs'!E20)/'Engine Inputs'!E20&gt;Config!$B$2,"📈 Up",IF((R20-'Engine Inputs'!E20)/'Engine Inputs'!E20&lt;-Config!$B$2,"📉 Down","➡ Stable"))))</f>
@@ -2348,13 +2348,13 @@
         </is>
       </c>
       <c r="D21" s="3" t="n">
-        <v>46247</v>
+        <v>46251</v>
       </c>
       <c r="E21" s="7" t="n">
-        <v>0</v>
+        <v>17.74</v>
       </c>
       <c r="F21" s="7" t="n">
-        <v>22.07</v>
+        <v>0</v>
       </c>
       <c r="G21" s="7">
         <f>E21-F21</f>
@@ -2365,36 +2365,36 @@
         <v/>
       </c>
       <c r="I21" s="7" t="n">
-        <v>20.9</v>
+        <v>0</v>
       </c>
       <c r="J21" s="6" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K21" s="6" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="L21" s="5">
         <f>IF(K21=0,"",(J21-K21)/K21)</f>
         <v/>
       </c>
       <c r="M21" s="6" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="N21" s="6" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="O21" s="7">
         <f>IF(J21=0,"",E21/J21)</f>
         <v/>
       </c>
       <c r="P21" s="6" t="n">
-        <v>193</v>
+        <v>200</v>
       </c>
       <c r="Q21" s="6" t="n">
-        <v>193</v>
+        <v>200</v>
       </c>
       <c r="R21" s="7" t="n">
-        <v>0</v>
+        <v>12.49</v>
       </c>
       <c r="S21" s="2">
         <f>IF(AND('Engine Inputs'!E21=0,R21=0),"",IF('Engine Inputs'!E21=0,"📈 Up",IF((R21-'Engine Inputs'!E21)/'Engine Inputs'!E21&gt;Config!$B$2,"📈 Up",IF((R21-'Engine Inputs'!E21)/'Engine Inputs'!E21&lt;-Config!$B$2,"📉 Down","➡ Stable"))))</f>
@@ -2437,7 +2437,7 @@
         </is>
       </c>
       <c r="D22" s="3" t="n">
-        <v>46247</v>
+        <v>46251</v>
       </c>
       <c r="E22" s="10" t="n">
         <v>0</v>
@@ -2454,7 +2454,7 @@
         <v/>
       </c>
       <c r="I22" s="10" t="n">
-        <v>44.67</v>
+        <v>0</v>
       </c>
       <c r="J22" s="6" t="n">
         <v>0</v>
@@ -2467,7 +2467,7 @@
         <v/>
       </c>
       <c r="M22" s="6" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="N22" s="6" t="n">
         <v>0</v>
@@ -2526,7 +2526,7 @@
         </is>
       </c>
       <c r="D23" s="3" t="n">
-        <v>46247</v>
+        <v>46251</v>
       </c>
       <c r="E23" s="7" t="n">
         <v>0</v>
@@ -2615,10 +2615,10 @@
         </is>
       </c>
       <c r="D24" s="3" t="n">
-        <v>46247</v>
+        <v>46251</v>
       </c>
       <c r="E24" s="7" t="n">
-        <v>0</v>
+        <v>20.89</v>
       </c>
       <c r="F24" s="7" t="n">
         <v>0</v>
@@ -2632,10 +2632,10 @@
         <v/>
       </c>
       <c r="I24" s="7" t="n">
-        <v>0</v>
+        <v>28.67</v>
       </c>
       <c r="J24" s="6" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K24" s="6" t="n">
         <v>0</v>
@@ -2645,10 +2645,10 @@
         <v/>
       </c>
       <c r="M24" s="6" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="N24" s="6" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="O24" s="7">
         <f>IF(J24=0,"",E24/J24)</f>
@@ -2661,7 +2661,7 @@
         <v>151</v>
       </c>
       <c r="R24" s="7" t="n">
-        <v>0</v>
+        <v>12.89</v>
       </c>
       <c r="S24" s="2">
         <f>IF(AND('Engine Inputs'!E24=0,R24=0),"",IF('Engine Inputs'!E24=0,"📈 Up",IF((R24-'Engine Inputs'!E24)/'Engine Inputs'!E24&gt;Config!$B$2,"📈 Up",IF((R24-'Engine Inputs'!E24)/'Engine Inputs'!E24&lt;-Config!$B$2,"📉 Down","➡ Stable"))))</f>
@@ -2704,7 +2704,7 @@
         </is>
       </c>
       <c r="D25" s="3" t="n">
-        <v>46247</v>
+        <v>46251</v>
       </c>
       <c r="E25" s="10" t="n">
         <v>0</v>
@@ -2793,7 +2793,7 @@
         </is>
       </c>
       <c r="D26" s="3" t="n">
-        <v>46247</v>
+        <v>46251</v>
       </c>
       <c r="E26" s="7" t="n">
         <v>0</v>
@@ -2882,13 +2882,13 @@
         </is>
       </c>
       <c r="D27" s="3" t="n">
-        <v>46247</v>
+        <v>46251</v>
       </c>
       <c r="E27" s="4" t="n">
-        <v>0</v>
+        <v>17.52</v>
       </c>
       <c r="F27" s="4" t="n">
-        <v>0</v>
+        <v>12.96</v>
       </c>
       <c r="G27" s="4">
         <f>E27-F27</f>
@@ -2902,10 +2902,10 @@
         <v>0</v>
       </c>
       <c r="J27" s="6" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K27" s="6" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L27" s="5">
         <f>IF(K27=0,"",(J27-K27)/K27)</f>
@@ -2915,7 +2915,7 @@
         <v>0</v>
       </c>
       <c r="N27" s="6" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="O27" s="4">
         <f>IF(J27=0,"",E27/J27)</f>
@@ -2928,7 +2928,7 @@
         <v>65</v>
       </c>
       <c r="R27" s="4" t="n">
-        <v>0</v>
+        <v>17.52</v>
       </c>
       <c r="S27" s="2">
         <f>IF(AND('Engine Inputs'!E27=0,R27=0),"",IF('Engine Inputs'!E27=0,"📈 Up",IF((R27-'Engine Inputs'!E27)/'Engine Inputs'!E27&gt;Config!$B$2,"📈 Up",IF((R27-'Engine Inputs'!E27)/'Engine Inputs'!E27&lt;-Config!$B$2,"📉 Down","➡ Stable"))))</f>
@@ -2971,7 +2971,7 @@
         </is>
       </c>
       <c r="D28" s="3" t="n">
-        <v>46247</v>
+        <v>46251</v>
       </c>
       <c r="E28" s="9" t="n">
         <v>0</v>
@@ -3060,7 +3060,7 @@
         </is>
       </c>
       <c r="D29" s="3" t="n">
-        <v>46247</v>
+        <v>46251</v>
       </c>
       <c r="E29" s="7" t="n">
         <v>0</v>
@@ -3149,7 +3149,7 @@
         </is>
       </c>
       <c r="D30" s="3" t="n">
-        <v>46247</v>
+        <v>46251</v>
       </c>
       <c r="E30" s="7" t="n">
         <v>0</v>
@@ -3238,7 +3238,7 @@
         </is>
       </c>
       <c r="D31" s="3" t="n">
-        <v>46247</v>
+        <v>46251</v>
       </c>
       <c r="E31" s="7" t="n">
         <v>0</v>
@@ -3327,7 +3327,7 @@
         </is>
       </c>
       <c r="D32" s="3" t="n">
-        <v>46247</v>
+        <v>46251</v>
       </c>
       <c r="E32" s="4" t="n">
         <v>0</v>
@@ -3416,7 +3416,7 @@
         </is>
       </c>
       <c r="D33" s="3" t="n">
-        <v>46247</v>
+        <v>46251</v>
       </c>
       <c r="E33" s="7" t="n">
         <v>0</v>
@@ -3521,7 +3521,7 @@
         </is>
       </c>
       <c r="B2" s="12" t="n">
-        <v>46247</v>
+        <v>46251</v>
       </c>
     </row>
     <row r="3">
@@ -3531,7 +3531,7 @@
         </is>
       </c>
       <c r="B3" s="12" t="n">
-        <v>46248</v>
+        <v>46252</v>
       </c>
     </row>
     <row r="5">
@@ -3943,12 +3943,12 @@
       </c>
       <c r="D1" s="13" t="inlineStr">
         <is>
-          <t>PH Sales 2026-08-12</t>
+          <t>PH Sales 2026-08-16</t>
         </is>
       </c>
       <c r="E1" s="13" t="inlineStr">
         <is>
-          <t>AH Sales 2026-08-12</t>
+          <t>AH Sales 2026-08-16</t>
         </is>
       </c>
       <c r="F1" s="15" t="inlineStr">
@@ -3974,10 +3974,10 @@
         </is>
       </c>
       <c r="D2" s="16" t="n">
-        <v>374.56</v>
+        <v>582.95</v>
       </c>
       <c r="E2" s="16" t="n">
-        <v>439.25</v>
+        <v>621.3200000000001</v>
       </c>
     </row>
     <row r="3">
@@ -3997,10 +3997,10 @@
         </is>
       </c>
       <c r="D3" s="16" t="n">
-        <v>81.38</v>
+        <v>157.43</v>
       </c>
       <c r="E3" s="16" t="n">
-        <v>147.06</v>
+        <v>146.03</v>
       </c>
     </row>
     <row r="4">
@@ -4020,10 +4020,10 @@
         </is>
       </c>
       <c r="D4" s="17" t="n">
-        <v>37.57</v>
+        <v>22.44</v>
       </c>
       <c r="E4" s="17" t="n">
-        <v>211.08</v>
+        <v>201.31</v>
       </c>
     </row>
     <row r="5">
@@ -4043,10 +4043,10 @@
         </is>
       </c>
       <c r="D5" s="16" t="n">
-        <v>73.70999999999999</v>
+        <v>130.93</v>
       </c>
       <c r="E5" s="16" t="n">
-        <v>88.81999999999999</v>
+        <v>106.36</v>
       </c>
     </row>
     <row r="6">
@@ -4066,10 +4066,10 @@
         </is>
       </c>
       <c r="D6" s="17" t="n">
-        <v>32.14</v>
+        <v>0</v>
       </c>
       <c r="E6" s="17" t="n">
-        <v>153.26</v>
+        <v>186.49</v>
       </c>
     </row>
     <row r="7">
@@ -4138,7 +4138,7 @@
         <v>0</v>
       </c>
       <c r="E9" s="16" t="n">
-        <v>304.11</v>
+        <v>197.39</v>
       </c>
     </row>
     <row r="10">
@@ -4158,10 +4158,10 @@
         </is>
       </c>
       <c r="D10" s="17" t="n">
-        <v>6.58</v>
+        <v>58.87</v>
       </c>
       <c r="E10" s="17" t="n">
-        <v>411.21</v>
+        <v>204.99</v>
       </c>
     </row>
     <row r="11">
@@ -4184,7 +4184,7 @@
         <v>0</v>
       </c>
       <c r="E11" s="16" t="n">
-        <v>36.99</v>
+        <v>85.44</v>
       </c>
     </row>
     <row r="12">
@@ -4204,10 +4204,10 @@
         </is>
       </c>
       <c r="D12" s="17" t="n">
-        <v>5.38</v>
+        <v>0</v>
       </c>
       <c r="E12" s="17" t="n">
-        <v>63.24</v>
+        <v>33.68</v>
       </c>
     </row>
     <row r="13">
@@ -4230,7 +4230,7 @@
         <v>0</v>
       </c>
       <c r="E13" s="16" t="n">
-        <v>113.02</v>
+        <v>107.38</v>
       </c>
     </row>
     <row r="14">
@@ -4253,7 +4253,7 @@
         <v>0</v>
       </c>
       <c r="E14" s="16" t="n">
-        <v>65.38</v>
+        <v>14.7</v>
       </c>
     </row>
     <row r="15">
@@ -4276,7 +4276,7 @@
         <v>0</v>
       </c>
       <c r="E15" s="17" t="n">
-        <v>0</v>
+        <v>9.41</v>
       </c>
     </row>
     <row r="16">
@@ -4299,7 +4299,7 @@
         <v>0</v>
       </c>
       <c r="E16" s="18" t="n">
-        <v>17.99</v>
+        <v>0</v>
       </c>
     </row>
     <row r="17">
@@ -4322,7 +4322,7 @@
         <v>0</v>
       </c>
       <c r="E17" s="18" t="n">
-        <v>0</v>
+        <v>14.3</v>
       </c>
     </row>
     <row r="18">
@@ -4345,7 +4345,7 @@
         <v>0</v>
       </c>
       <c r="E18" s="18" t="n">
-        <v>0</v>
+        <v>134.96</v>
       </c>
     </row>
     <row r="19">
@@ -4391,7 +4391,7 @@
         <v>0</v>
       </c>
       <c r="E20" s="16" t="n">
-        <v>7.89</v>
+        <v>0</v>
       </c>
     </row>
     <row r="21">
@@ -4414,7 +4414,7 @@
         <v>0</v>
       </c>
       <c r="E21" s="17" t="n">
-        <v>17.98</v>
+        <v>0</v>
       </c>
     </row>
     <row r="22">
@@ -4552,7 +4552,7 @@
         <v>0</v>
       </c>
       <c r="E27" s="16" t="n">
-        <v>0</v>
+        <v>12.96</v>
       </c>
     </row>
     <row r="28">
@@ -4806,7 +4806,7 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t xml:space="preserve">  Generated 2026-08-14.  "Today" = 2026-08-13.  "Yesterday" = 2026-08-12.  Same Day LY = 2025-08-13.</t>
+          <t xml:space="preserve">  Generated 2026-08-18.  "Today" = 2026-08-17.  "Yesterday" = 2026-08-16.  Same Day LY = 2025-08-17.</t>
         </is>
       </c>
     </row>
@@ -4851,7 +4851,7 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t xml:space="preserve">  Why not 'Completed' only: orders reach Completed about 2 days after purchase. On 2026-08-13</t>
+          <t xml:space="preserve">  Why not 'Completed' only: orders reach Completed about 2 days after purchase. On 2026-08-17</t>
         </is>
       </c>
     </row>
@@ -5162,7 +5162,7 @@
     <row r="72">
       <c r="A72" t="inlineStr">
         <is>
-          <t xml:space="preserve">  (2026-08-13 was a Thursday; 2025-08-13 was a Wednesday). Day-of-week effects are present in this comparison.</t>
+          <t xml:space="preserve">  (2026-08-17 was a Monday; 2025-08-17 was a Sunday). Day-of-week effects are present in this comparison.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
chore(dst): commit the 2026-08-19 scheduled run output
Output of the daily 09:05 job (ran 09:19), left uncommitted in the working tree.
Not a hand edit - the window rolled forward one day, anchor 2026-08-17 ->
2026-08-18, same 32 account x marketplace rows, same structure, refreshed
figures. Committing so the folder matches what the automation actually produced.
</commit_message>
<xml_diff>
--- a/development/abiraj_mini_aios_workbench/projects/PRJ-2026-015_daily-sales-track/evidence/final_outputs/REQ-17_daily-sales-track/REQ-17-D01_daily_sales_track.xlsx
+++ b/development/abiraj_mini_aios_workbench/projects/PRJ-2026-015_daily-sales-track/evidence/final_outputs/REQ-17_daily-sales-track/REQ-17-D01_daily_sales_track.xlsx
@@ -657,13 +657,13 @@
         </is>
       </c>
       <c r="D2" s="3" t="n">
-        <v>46251</v>
+        <v>46252</v>
       </c>
       <c r="E2" s="4" t="n">
-        <v>1122.21</v>
+        <v>1099.92</v>
       </c>
       <c r="F2" s="4" t="n">
-        <v>1160.45</v>
+        <v>1110.72</v>
       </c>
       <c r="G2" s="4">
         <f>E2-F2</f>
@@ -674,36 +674,36 @@
         <v/>
       </c>
       <c r="I2" s="4" t="n">
-        <v>928.1</v>
+        <v>1599.22</v>
       </c>
       <c r="J2" s="6" t="n">
-        <v>67</v>
+        <v>57</v>
       </c>
       <c r="K2" s="6" t="n">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="L2" s="5">
         <f>IF(K2=0,"",(J2-K2)/K2)</f>
         <v/>
       </c>
       <c r="M2" s="6" t="n">
-        <v>69</v>
+        <v>86</v>
       </c>
       <c r="N2" s="6" t="n">
-        <v>104</v>
+        <v>95</v>
       </c>
       <c r="O2" s="4">
         <f>IF(J2=0,"",E2/J2)</f>
         <v/>
       </c>
       <c r="P2" s="6" t="n">
-        <v>3062</v>
+        <v>3064</v>
       </c>
       <c r="Q2" s="6" t="n">
-        <v>1756</v>
+        <v>1758</v>
       </c>
       <c r="R2" s="4" t="n">
-        <v>603.2</v>
+        <v>656.29</v>
       </c>
       <c r="S2" s="2">
         <f>IF(AND('Engine Inputs'!E2=0,R2=0),"",IF('Engine Inputs'!E2=0,"📈 Up",IF((R2-'Engine Inputs'!E2)/'Engine Inputs'!E2&gt;Config!$B$2,"📈 Up",IF((R2-'Engine Inputs'!E2)/'Engine Inputs'!E2&lt;-Config!$B$2,"📉 Down","➡ Stable"))))</f>
@@ -713,7 +713,7 @@
         <v>1306</v>
       </c>
       <c r="U2" s="4" t="n">
-        <v>517.77</v>
+        <v>439.76</v>
       </c>
       <c r="V2" s="2">
         <f>IF(AND('Engine Inputs'!D2=0,U2=0),"",IF('Engine Inputs'!D2=0,"📈 Up",IF((U2-'Engine Inputs'!D2)/'Engine Inputs'!D2&gt;Config!$B$2,"📈 Up",IF((U2-'Engine Inputs'!D2)/'Engine Inputs'!D2&lt;-Config!$B$2,"📉 Down","➡ Stable"))))</f>
@@ -746,13 +746,13 @@
         </is>
       </c>
       <c r="D3" s="3" t="n">
-        <v>46251</v>
+        <v>46252</v>
       </c>
       <c r="E3" s="4" t="n">
-        <v>537.51</v>
+        <v>374.52</v>
       </c>
       <c r="F3" s="4" t="n">
-        <v>293.97</v>
+        <v>488.06</v>
       </c>
       <c r="G3" s="4">
         <f>E3-F3</f>
@@ -763,36 +763,36 @@
         <v/>
       </c>
       <c r="I3" s="4" t="n">
-        <v>764.91</v>
+        <v>481.24</v>
       </c>
       <c r="J3" s="6" t="n">
-        <v>33</v>
+        <v>25</v>
       </c>
       <c r="K3" s="6" t="n">
-        <v>19</v>
+        <v>32</v>
       </c>
       <c r="L3" s="5">
         <f>IF(K3=0,"",(J3-K3)/K3)</f>
         <v/>
       </c>
       <c r="M3" s="6" t="n">
-        <v>47</v>
+        <v>32</v>
       </c>
       <c r="N3" s="6" t="n">
-        <v>44</v>
+        <v>30</v>
       </c>
       <c r="O3" s="4">
         <f>IF(J3=0,"",E3/J3)</f>
         <v/>
       </c>
       <c r="P3" s="6" t="n">
-        <v>1699</v>
+        <v>1702</v>
       </c>
       <c r="Q3" s="6" t="n">
-        <v>1102</v>
+        <v>1105</v>
       </c>
       <c r="R3" s="4" t="n">
-        <v>306.32</v>
+        <v>151.51</v>
       </c>
       <c r="S3" s="2">
         <f>IF(AND('Engine Inputs'!E3=0,R3=0),"",IF('Engine Inputs'!E3=0,"📈 Up",IF((R3-'Engine Inputs'!E3)/'Engine Inputs'!E3&gt;Config!$B$2,"📈 Up",IF((R3-'Engine Inputs'!E3)/'Engine Inputs'!E3&lt;-Config!$B$2,"📉 Down","➡ Stable"))))</f>
@@ -802,7 +802,7 @@
         <v>597</v>
       </c>
       <c r="U3" s="4" t="n">
-        <v>237.96</v>
+        <v>234.39</v>
       </c>
       <c r="V3" s="2">
         <f>IF(AND('Engine Inputs'!D3=0,U3=0),"",IF('Engine Inputs'!D3=0,"📈 Up",IF((U3-'Engine Inputs'!D3)/'Engine Inputs'!D3&gt;Config!$B$2,"📈 Up",IF((U3-'Engine Inputs'!D3)/'Engine Inputs'!D3&lt;-Config!$B$2,"📉 Down","➡ Stable"))))</f>
@@ -835,13 +835,13 @@
         </is>
       </c>
       <c r="D4" s="3" t="n">
-        <v>46251</v>
+        <v>46252</v>
       </c>
       <c r="E4" s="7" t="n">
+        <v>96.8</v>
+      </c>
+      <c r="F4" s="7" t="n">
         <v>302.99</v>
-      </c>
-      <c r="F4" s="7" t="n">
-        <v>320.86</v>
       </c>
       <c r="G4" s="7">
         <f>E4-F4</f>
@@ -852,23 +852,23 @@
         <v/>
       </c>
       <c r="I4" s="7" t="n">
-        <v>767.77</v>
+        <v>315.86</v>
       </c>
       <c r="J4" s="6" t="n">
+        <v>4</v>
+      </c>
+      <c r="K4" s="6" t="n">
         <v>13</v>
-      </c>
-      <c r="K4" s="6" t="n">
-        <v>12</v>
       </c>
       <c r="L4" s="5">
         <f>IF(K4=0,"",(J4-K4)/K4)</f>
         <v/>
       </c>
       <c r="M4" s="6" t="n">
-        <v>25</v>
+        <v>13</v>
       </c>
       <c r="N4" s="6" t="n">
-        <v>16</v>
+        <v>5</v>
       </c>
       <c r="O4" s="7">
         <f>IF(J4=0,"",E4/J4)</f>
@@ -881,7 +881,7 @@
         <v>1221</v>
       </c>
       <c r="R4" s="7" t="n">
-        <v>199.69</v>
+        <v>65.90000000000001</v>
       </c>
       <c r="S4" s="2">
         <f>IF(AND('Engine Inputs'!E4=0,R4=0),"",IF('Engine Inputs'!E4=0,"📈 Up",IF((R4-'Engine Inputs'!E4)/'Engine Inputs'!E4&gt;Config!$B$2,"📈 Up",IF((R4-'Engine Inputs'!E4)/'Engine Inputs'!E4&lt;-Config!$B$2,"📉 Down","➡ Stable"))))</f>
@@ -891,7 +891,7 @@
         <v>232</v>
       </c>
       <c r="U4" s="7" t="n">
-        <v>3.78</v>
+        <v>0</v>
       </c>
       <c r="V4" s="2">
         <f>IF(AND('Engine Inputs'!D4=0,U4=0),"",IF('Engine Inputs'!D4=0,"📈 Up",IF((U4-'Engine Inputs'!D4)/'Engine Inputs'!D4&gt;Config!$B$2,"📈 Up",IF((U4-'Engine Inputs'!D4)/'Engine Inputs'!D4&lt;-Config!$B$2,"📉 Down","➡ Stable"))))</f>
@@ -924,13 +924,13 @@
         </is>
       </c>
       <c r="D5" s="3" t="n">
-        <v>46251</v>
+        <v>46252</v>
       </c>
       <c r="E5" s="4" t="n">
+        <v>194.94</v>
+      </c>
+      <c r="F5" s="4" t="n">
         <v>320.64</v>
-      </c>
-      <c r="F5" s="4" t="n">
-        <v>234.77</v>
       </c>
       <c r="G5" s="4">
         <f>E5-F5</f>
@@ -941,36 +941,36 @@
         <v/>
       </c>
       <c r="I5" s="4" t="n">
-        <v>203.52</v>
+        <v>355.25</v>
       </c>
       <c r="J5" s="6" t="n">
+        <v>12</v>
+      </c>
+      <c r="K5" s="6" t="n">
         <v>18</v>
-      </c>
-      <c r="K5" s="6" t="n">
-        <v>15</v>
       </c>
       <c r="L5" s="5">
         <f>IF(K5=0,"",(J5-K5)/K5)</f>
         <v/>
       </c>
       <c r="M5" s="6" t="n">
-        <v>14</v>
+        <v>17</v>
       </c>
       <c r="N5" s="6" t="n">
-        <v>34</v>
+        <v>15</v>
       </c>
       <c r="O5" s="4">
         <f>IF(J5=0,"",E5/J5)</f>
         <v/>
       </c>
       <c r="P5" s="6" t="n">
-        <v>1214</v>
+        <v>1216</v>
       </c>
       <c r="Q5" s="6" t="n">
-        <v>744</v>
+        <v>746</v>
       </c>
       <c r="R5" s="4" t="n">
-        <v>234.1</v>
+        <v>92.94</v>
       </c>
       <c r="S5" s="2">
         <f>IF(AND('Engine Inputs'!E5=0,R5=0),"",IF('Engine Inputs'!E5=0,"📈 Up",IF((R5-'Engine Inputs'!E5)/'Engine Inputs'!E5&gt;Config!$B$2,"📈 Up",IF((R5-'Engine Inputs'!E5)/'Engine Inputs'!E5&lt;-Config!$B$2,"📉 Down","➡ Stable"))))</f>
@@ -980,7 +980,7 @@
         <v>470</v>
       </c>
       <c r="U5" s="4" t="n">
-        <v>87.39</v>
+        <v>100.81</v>
       </c>
       <c r="V5" s="2">
         <f>IF(AND('Engine Inputs'!D5=0,U5=0),"",IF('Engine Inputs'!D5=0,"📈 Up",IF((U5-'Engine Inputs'!D5)/'Engine Inputs'!D5&gt;Config!$B$2,"📈 Up",IF((U5-'Engine Inputs'!D5)/'Engine Inputs'!D5&lt;-Config!$B$2,"📉 Down","➡ Stable"))))</f>
@@ -1013,13 +1013,13 @@
         </is>
       </c>
       <c r="D6" s="3" t="n">
-        <v>46251</v>
+        <v>46252</v>
       </c>
       <c r="E6" s="7" t="n">
+        <v>121.13</v>
+      </c>
+      <c r="F6" s="7" t="n">
         <v>170.81</v>
-      </c>
-      <c r="F6" s="7" t="n">
-        <v>211.06</v>
       </c>
       <c r="G6" s="7">
         <f>E6-F6</f>
@@ -1030,7 +1030,7 @@
         <v/>
       </c>
       <c r="I6" s="7" t="n">
-        <v>337.65</v>
+        <v>221.54</v>
       </c>
       <c r="J6" s="6" t="n">
         <v>6</v>
@@ -1043,23 +1043,23 @@
         <v/>
       </c>
       <c r="M6" s="6" t="n">
-        <v>19</v>
+        <v>15</v>
       </c>
       <c r="N6" s="6" t="n">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="O6" s="7">
         <f>IF(J6=0,"",E6/J6)</f>
         <v/>
       </c>
       <c r="P6" s="6" t="n">
-        <v>670</v>
+        <v>671</v>
       </c>
       <c r="Q6" s="6" t="n">
-        <v>581</v>
+        <v>582</v>
       </c>
       <c r="R6" s="7" t="n">
-        <v>128.94</v>
+        <v>89.63</v>
       </c>
       <c r="S6" s="2">
         <f>IF(AND('Engine Inputs'!E6=0,R6=0),"",IF('Engine Inputs'!E6=0,"📈 Up",IF((R6-'Engine Inputs'!E6)/'Engine Inputs'!E6&gt;Config!$B$2,"📈 Up",IF((R6-'Engine Inputs'!E6)/'Engine Inputs'!E6&lt;-Config!$B$2,"📉 Down","➡ Stable"))))</f>
@@ -1069,7 +1069,7 @@
         <v>89</v>
       </c>
       <c r="U6" s="7" t="n">
-        <v>14.99</v>
+        <v>0</v>
       </c>
       <c r="V6" s="2">
         <f>IF(AND('Engine Inputs'!D6=0,U6=0),"",IF('Engine Inputs'!D6=0,"📈 Up",IF((U6-'Engine Inputs'!D6)/'Engine Inputs'!D6&gt;Config!$B$2,"📈 Up",IF((U6-'Engine Inputs'!D6)/'Engine Inputs'!D6&lt;-Config!$B$2,"📉 Down","➡ Stable"))))</f>
@@ -1102,7 +1102,7 @@
         </is>
       </c>
       <c r="D7" s="3" t="n">
-        <v>46251</v>
+        <v>46252</v>
       </c>
       <c r="E7" s="7" t="n">
         <v>0</v>
@@ -1191,7 +1191,7 @@
         </is>
       </c>
       <c r="D8" s="3" t="n">
-        <v>46251</v>
+        <v>46252</v>
       </c>
       <c r="E8" s="7" t="n">
         <v>0</v>
@@ -1280,13 +1280,13 @@
         </is>
       </c>
       <c r="D9" s="3" t="n">
-        <v>46251</v>
+        <v>46252</v>
       </c>
       <c r="E9" s="4" t="n">
+        <v>219.92</v>
+      </c>
+      <c r="F9" s="4" t="n">
         <v>223.61</v>
-      </c>
-      <c r="F9" s="4" t="n">
-        <v>164.5</v>
       </c>
       <c r="G9" s="4">
         <f>E9-F9</f>
@@ -1297,23 +1297,23 @@
         <v/>
       </c>
       <c r="I9" s="4" t="n">
-        <v>162.52</v>
+        <v>314.91</v>
       </c>
       <c r="J9" s="6" t="n">
+        <v>13</v>
+      </c>
+      <c r="K9" s="6" t="n">
         <v>16</v>
-      </c>
-      <c r="K9" s="6" t="n">
-        <v>7</v>
       </c>
       <c r="L9" s="5">
         <f>IF(K9=0,"",(J9-K9)/K9)</f>
         <v/>
       </c>
       <c r="M9" s="6" t="n">
-        <v>15</v>
+        <v>19</v>
       </c>
       <c r="N9" s="6" t="n">
-        <v>19</v>
+        <v>13</v>
       </c>
       <c r="O9" s="4">
         <f>IF(J9=0,"",E9/J9)</f>
@@ -1326,7 +1326,7 @@
         <v>579</v>
       </c>
       <c r="R9" s="4" t="n">
-        <v>223.61</v>
+        <v>219.92</v>
       </c>
       <c r="S9" s="2">
         <f>IF(AND('Engine Inputs'!E9=0,R9=0),"",IF('Engine Inputs'!E9=0,"📈 Up",IF((R9-'Engine Inputs'!E9)/'Engine Inputs'!E9&gt;Config!$B$2,"📈 Up",IF((R9-'Engine Inputs'!E9)/'Engine Inputs'!E9&lt;-Config!$B$2,"📉 Down","➡ Stable"))))</f>
@@ -1369,13 +1369,13 @@
         </is>
       </c>
       <c r="D10" s="3" t="n">
-        <v>46251</v>
+        <v>46252</v>
       </c>
       <c r="E10" s="7" t="n">
+        <v>346.21</v>
+      </c>
+      <c r="F10" s="7" t="n">
         <v>288.24</v>
-      </c>
-      <c r="F10" s="7" t="n">
-        <v>323.05</v>
       </c>
       <c r="G10" s="7">
         <f>E10-F10</f>
@@ -1386,23 +1386,23 @@
         <v/>
       </c>
       <c r="I10" s="7" t="n">
-        <v>240.18</v>
+        <v>415.37</v>
       </c>
       <c r="J10" s="6" t="n">
+        <v>13</v>
+      </c>
+      <c r="K10" s="6" t="n">
         <v>11</v>
-      </c>
-      <c r="K10" s="6" t="n">
-        <v>13</v>
       </c>
       <c r="L10" s="5">
         <f>IF(K10=0,"",(J10-K10)/K10)</f>
         <v/>
       </c>
       <c r="M10" s="6" t="n">
-        <v>13</v>
+        <v>23</v>
       </c>
       <c r="N10" s="6" t="n">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="O10" s="7">
         <f>IF(J10=0,"",E10/J10)</f>
@@ -1415,7 +1415,7 @@
         <v>467</v>
       </c>
       <c r="R10" s="7" t="n">
-        <v>207.36</v>
+        <v>287.71</v>
       </c>
       <c r="S10" s="2">
         <f>IF(AND('Engine Inputs'!E10=0,R10=0),"",IF('Engine Inputs'!E10=0,"📈 Up",IF((R10-'Engine Inputs'!E10)/'Engine Inputs'!E10&gt;Config!$B$2,"📈 Up",IF((R10-'Engine Inputs'!E10)/'Engine Inputs'!E10&lt;-Config!$B$2,"📉 Down","➡ Stable"))))</f>
@@ -1425,7 +1425,7 @@
         <v>93</v>
       </c>
       <c r="U10" s="7" t="n">
-        <v>37.27</v>
+        <v>0</v>
       </c>
       <c r="V10" s="2">
         <f>IF(AND('Engine Inputs'!D10=0,U10=0),"",IF('Engine Inputs'!D10=0,"📈 Up",IF((U10-'Engine Inputs'!D10)/'Engine Inputs'!D10&gt;Config!$B$2,"📈 Up",IF((U10-'Engine Inputs'!D10)/'Engine Inputs'!D10&lt;-Config!$B$2,"📉 Down","➡ Stable"))))</f>
@@ -1458,13 +1458,13 @@
         </is>
       </c>
       <c r="D11" s="3" t="n">
-        <v>46251</v>
+        <v>46252</v>
       </c>
       <c r="E11" s="4" t="n">
+        <v>110.16</v>
+      </c>
+      <c r="F11" s="4" t="n">
         <v>111.89</v>
-      </c>
-      <c r="F11" s="4" t="n">
-        <v>78.98999999999999</v>
       </c>
       <c r="G11" s="4">
         <f>E11-F11</f>
@@ -1475,23 +1475,23 @@
         <v/>
       </c>
       <c r="I11" s="4" t="n">
-        <v>106.52</v>
+        <v>84.56999999999999</v>
       </c>
       <c r="J11" s="6" t="n">
+        <v>6</v>
+      </c>
+      <c r="K11" s="6" t="n">
         <v>8</v>
-      </c>
-      <c r="K11" s="6" t="n">
-        <v>7</v>
       </c>
       <c r="L11" s="5">
         <f>IF(K11=0,"",(J11-K11)/K11)</f>
         <v/>
       </c>
       <c r="M11" s="6" t="n">
-        <v>15</v>
+        <v>6</v>
       </c>
       <c r="N11" s="6" t="n">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="O11" s="4">
         <f>IF(J11=0,"",E11/J11)</f>
@@ -1504,7 +1504,7 @@
         <v>509</v>
       </c>
       <c r="R11" s="4" t="n">
-        <v>115.44</v>
+        <v>117.55</v>
       </c>
       <c r="S11" s="2">
         <f>IF(AND('Engine Inputs'!E11=0,R11=0),"",IF('Engine Inputs'!E11=0,"📈 Up",IF((R11-'Engine Inputs'!E11)/'Engine Inputs'!E11&gt;Config!$B$2,"📈 Up",IF((R11-'Engine Inputs'!E11)/'Engine Inputs'!E11&lt;-Config!$B$2,"📉 Down","➡ Stable"))))</f>
@@ -1547,13 +1547,13 @@
         </is>
       </c>
       <c r="D12" s="3" t="n">
-        <v>46251</v>
+        <v>46252</v>
       </c>
       <c r="E12" s="7" t="n">
+        <v>77.12</v>
+      </c>
+      <c r="F12" s="7" t="n">
         <v>14.14</v>
-      </c>
-      <c r="F12" s="7" t="n">
-        <v>60.28</v>
       </c>
       <c r="G12" s="7">
         <f>E12-F12</f>
@@ -1564,23 +1564,23 @@
         <v/>
       </c>
       <c r="I12" s="7" t="n">
-        <v>208.28</v>
+        <v>83.76000000000001</v>
       </c>
       <c r="J12" s="6" t="n">
+        <v>4</v>
+      </c>
+      <c r="K12" s="6" t="n">
         <v>1</v>
-      </c>
-      <c r="K12" s="6" t="n">
-        <v>4</v>
       </c>
       <c r="L12" s="5">
         <f>IF(K12=0,"",(J12-K12)/K12)</f>
         <v/>
       </c>
       <c r="M12" s="6" t="n">
-        <v>10</v>
+        <v>7</v>
       </c>
       <c r="N12" s="6" t="n">
-        <v>1</v>
+        <v>7</v>
       </c>
       <c r="O12" s="7">
         <f>IF(J12=0,"",E12/J12)</f>
@@ -1593,7 +1593,7 @@
         <v>454</v>
       </c>
       <c r="R12" s="7" t="n">
-        <v>7.47</v>
+        <v>50.03</v>
       </c>
       <c r="S12" s="2">
         <f>IF(AND('Engine Inputs'!E12=0,R12=0),"",IF('Engine Inputs'!E12=0,"📈 Up",IF((R12-'Engine Inputs'!E12)/'Engine Inputs'!E12&gt;Config!$B$2,"📈 Up",IF((R12-'Engine Inputs'!E12)/'Engine Inputs'!E12&lt;-Config!$B$2,"📉 Down","➡ Stable"))))</f>
@@ -1636,13 +1636,13 @@
         </is>
       </c>
       <c r="D13" s="3" t="n">
-        <v>46251</v>
+        <v>46252</v>
       </c>
       <c r="E13" s="4" t="n">
+        <v>297.6</v>
+      </c>
+      <c r="F13" s="4" t="n">
         <v>6.99</v>
-      </c>
-      <c r="F13" s="4" t="n">
-        <v>102.12</v>
       </c>
       <c r="G13" s="4">
         <f>E13-F13</f>
@@ -1653,23 +1653,23 @@
         <v/>
       </c>
       <c r="I13" s="4" t="n">
-        <v>78.14</v>
+        <v>159.61</v>
       </c>
       <c r="J13" s="6" t="n">
+        <v>10</v>
+      </c>
+      <c r="K13" s="6" t="n">
         <v>1</v>
-      </c>
-      <c r="K13" s="6" t="n">
-        <v>9</v>
       </c>
       <c r="L13" s="5">
         <f>IF(K13=0,"",(J13-K13)/K13)</f>
         <v/>
       </c>
       <c r="M13" s="6" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="N13" s="6" t="n">
-        <v>1</v>
+        <v>27</v>
       </c>
       <c r="O13" s="4">
         <f>IF(J13=0,"",E13/J13)</f>
@@ -1682,7 +1682,7 @@
         <v>487</v>
       </c>
       <c r="R13" s="4" t="n">
-        <v>6.99</v>
+        <v>324.09</v>
       </c>
       <c r="S13" s="2">
         <f>IF(AND('Engine Inputs'!E13=0,R13=0),"",IF('Engine Inputs'!E13=0,"📈 Up",IF((R13-'Engine Inputs'!E13)/'Engine Inputs'!E13&gt;Config!$B$2,"📈 Up",IF((R13-'Engine Inputs'!E13)/'Engine Inputs'!E13&lt;-Config!$B$2,"📉 Down","➡ Stable"))))</f>
@@ -1725,13 +1725,13 @@
         </is>
       </c>
       <c r="D14" s="3" t="n">
-        <v>46251</v>
+        <v>46252</v>
       </c>
       <c r="E14" s="4" t="n">
+        <v>12.89</v>
+      </c>
+      <c r="F14" s="4" t="n">
         <v>90.76000000000001</v>
-      </c>
-      <c r="F14" s="4" t="n">
-        <v>14.7</v>
       </c>
       <c r="G14" s="4">
         <f>E14-F14</f>
@@ -1742,23 +1742,23 @@
         <v/>
       </c>
       <c r="I14" s="4" t="n">
-        <v>32.4</v>
+        <v>97.73999999999999</v>
       </c>
       <c r="J14" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="K14" s="6" t="n">
         <v>3</v>
-      </c>
-      <c r="K14" s="6" t="n">
-        <v>1</v>
       </c>
       <c r="L14" s="5">
         <f>IF(K14=0,"",(J14-K14)/K14)</f>
         <v/>
       </c>
       <c r="M14" s="6" t="n">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="N14" s="6" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="O14" s="4">
         <f>IF(J14=0,"",E14/J14)</f>
@@ -1771,7 +1771,7 @@
         <v>435</v>
       </c>
       <c r="R14" s="4" t="n">
-        <v>90.76000000000001</v>
+        <v>12.89</v>
       </c>
       <c r="S14" s="2">
         <f>IF(AND('Engine Inputs'!E14=0,R14=0),"",IF('Engine Inputs'!E14=0,"📈 Up",IF((R14-'Engine Inputs'!E14)/'Engine Inputs'!E14&gt;Config!$B$2,"📈 Up",IF((R14-'Engine Inputs'!E14)/'Engine Inputs'!E14&lt;-Config!$B$2,"📉 Down","➡ Stable"))))</f>
@@ -1814,13 +1814,13 @@
         </is>
       </c>
       <c r="D15" s="3" t="n">
-        <v>46251</v>
+        <v>46252</v>
       </c>
       <c r="E15" s="7" t="n">
         <v>0</v>
       </c>
       <c r="F15" s="7" t="n">
-        <v>26.73</v>
+        <v>0</v>
       </c>
       <c r="G15" s="7">
         <f>E15-F15</f>
@@ -1831,20 +1831,20 @@
         <v/>
       </c>
       <c r="I15" s="7" t="n">
-        <v>0</v>
+        <v>40.33</v>
       </c>
       <c r="J15" s="6" t="n">
         <v>0</v>
       </c>
       <c r="K15" s="6" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="L15" s="5">
         <f>IF(K15=0,"",(J15-K15)/K15)</f>
         <v/>
       </c>
       <c r="M15" s="6" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="N15" s="6" t="n">
         <v>0</v>
@@ -1903,7 +1903,7 @@
         </is>
       </c>
       <c r="D16" s="3" t="n">
-        <v>46251</v>
+        <v>46252</v>
       </c>
       <c r="E16" s="9" t="n">
         <v>0</v>
@@ -1920,7 +1920,7 @@
         <v/>
       </c>
       <c r="I16" s="9" t="n">
-        <v>0</v>
+        <v>70.98</v>
       </c>
       <c r="J16" s="6" t="n">
         <v>0</v>
@@ -1933,7 +1933,7 @@
         <v/>
       </c>
       <c r="M16" s="6" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="N16" s="6" t="n">
         <v>0</v>
@@ -1992,13 +1992,13 @@
         </is>
       </c>
       <c r="D17" s="3" t="n">
-        <v>46251</v>
+        <v>46252</v>
       </c>
       <c r="E17" s="9" t="n">
+        <v>33.38</v>
+      </c>
+      <c r="F17" s="9" t="n">
         <v>28.47</v>
-      </c>
-      <c r="F17" s="9" t="n">
-        <v>15.19</v>
       </c>
       <c r="G17" s="9">
         <f>E17-F17</f>
@@ -2038,7 +2038,7 @@
         <v>377</v>
       </c>
       <c r="R17" s="9" t="n">
-        <v>26.99</v>
+        <v>31.49</v>
       </c>
       <c r="S17" s="2">
         <f>IF(AND('Engine Inputs'!E17=0,R17=0),"",IF('Engine Inputs'!E17=0,"📈 Up",IF((R17-'Engine Inputs'!E17)/'Engine Inputs'!E17&gt;Config!$B$2,"📈 Up",IF((R17-'Engine Inputs'!E17)/'Engine Inputs'!E17&lt;-Config!$B$2,"📉 Down","➡ Stable"))))</f>
@@ -2081,13 +2081,13 @@
         </is>
       </c>
       <c r="D18" s="3" t="n">
-        <v>46251</v>
+        <v>46252</v>
       </c>
       <c r="E18" s="9" t="n">
+        <v>17.17</v>
+      </c>
+      <c r="F18" s="9" t="n">
         <v>23.44</v>
-      </c>
-      <c r="F18" s="9" t="n">
-        <v>145.04</v>
       </c>
       <c r="G18" s="9">
         <f>E18-F18</f>
@@ -2098,20 +2098,20 @@
         <v/>
       </c>
       <c r="I18" s="9" t="n">
-        <v>0</v>
+        <v>27.86</v>
       </c>
       <c r="J18" s="6" t="n">
         <v>1</v>
       </c>
       <c r="K18" s="6" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="L18" s="5">
         <f>IF(K18=0,"",(J18-K18)/K18)</f>
         <v/>
       </c>
       <c r="M18" s="6" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="N18" s="6" t="n">
         <v>1</v>
@@ -2127,7 +2127,7 @@
         <v>329</v>
       </c>
       <c r="R18" s="9" t="n">
-        <v>21.5</v>
+        <v>16.19</v>
       </c>
       <c r="S18" s="2">
         <f>IF(AND('Engine Inputs'!E18=0,R18=0),"",IF('Engine Inputs'!E18=0,"📈 Up",IF((R18-'Engine Inputs'!E18)/'Engine Inputs'!E18&gt;Config!$B$2,"📈 Up",IF((R18-'Engine Inputs'!E18)/'Engine Inputs'!E18&lt;-Config!$B$2,"📉 Down","➡ Stable"))))</f>
@@ -2170,10 +2170,10 @@
         </is>
       </c>
       <c r="D19" s="3" t="n">
-        <v>46251</v>
+        <v>46252</v>
       </c>
       <c r="E19" s="7" t="n">
-        <v>0</v>
+        <v>43.31</v>
       </c>
       <c r="F19" s="7" t="n">
         <v>0</v>
@@ -2187,10 +2187,10 @@
         <v/>
       </c>
       <c r="I19" s="7" t="n">
-        <v>117.93</v>
+        <v>72.04000000000001</v>
       </c>
       <c r="J19" s="6" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="K19" s="6" t="n">
         <v>0</v>
@@ -2203,7 +2203,7 @@
         <v>6</v>
       </c>
       <c r="N19" s="6" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="O19" s="7">
         <f>IF(J19=0,"",E19/J19)</f>
@@ -2216,7 +2216,7 @@
         <v>301</v>
       </c>
       <c r="R19" s="7" t="n">
-        <v>0</v>
+        <v>23.15</v>
       </c>
       <c r="S19" s="2">
         <f>IF(AND('Engine Inputs'!E19=0,R19=0),"",IF('Engine Inputs'!E19=0,"📈 Up",IF((R19-'Engine Inputs'!E19)/'Engine Inputs'!E19&gt;Config!$B$2,"📈 Up",IF((R19-'Engine Inputs'!E19)/'Engine Inputs'!E19&lt;-Config!$B$2,"📉 Down","➡ Stable"))))</f>
@@ -2259,13 +2259,13 @@
         </is>
       </c>
       <c r="D20" s="3" t="n">
-        <v>46251</v>
+        <v>46252</v>
       </c>
       <c r="E20" s="4" t="n">
+        <v>15.96</v>
+      </c>
+      <c r="F20" s="4" t="n">
         <v>34.88</v>
-      </c>
-      <c r="F20" s="4" t="n">
-        <v>0</v>
       </c>
       <c r="G20" s="4">
         <f>E20-F20</f>
@@ -2276,20 +2276,20 @@
         <v/>
       </c>
       <c r="I20" s="4" t="n">
-        <v>71.70999999999999</v>
+        <v>10.18</v>
       </c>
       <c r="J20" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="K20" s="6" t="n">
         <v>2</v>
-      </c>
-      <c r="K20" s="6" t="n">
-        <v>0</v>
       </c>
       <c r="L20" s="5">
         <f>IF(K20=0,"",(J20-K20)/K20)</f>
         <v/>
       </c>
       <c r="M20" s="6" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="N20" s="6" t="n">
         <v>2</v>
@@ -2305,7 +2305,7 @@
         <v>266</v>
       </c>
       <c r="R20" s="4" t="n">
-        <v>34.88</v>
+        <v>15.96</v>
       </c>
       <c r="S20" s="2">
         <f>IF(AND('Engine Inputs'!E20=0,R20=0),"",IF('Engine Inputs'!E20=0,"📈 Up",IF((R20-'Engine Inputs'!E20)/'Engine Inputs'!E20&gt;Config!$B$2,"📈 Up",IF((R20-'Engine Inputs'!E20)/'Engine Inputs'!E20&lt;-Config!$B$2,"📉 Down","➡ Stable"))))</f>
@@ -2348,13 +2348,13 @@
         </is>
       </c>
       <c r="D21" s="3" t="n">
-        <v>46251</v>
+        <v>46252</v>
       </c>
       <c r="E21" s="7" t="n">
+        <v>9.630000000000001</v>
+      </c>
+      <c r="F21" s="7" t="n">
         <v>17.74</v>
-      </c>
-      <c r="F21" s="7" t="n">
-        <v>0</v>
       </c>
       <c r="G21" s="7">
         <f>E21-F21</f>
@@ -2365,20 +2365,20 @@
         <v/>
       </c>
       <c r="I21" s="7" t="n">
-        <v>0</v>
+        <v>28.55</v>
       </c>
       <c r="J21" s="6" t="n">
         <v>1</v>
       </c>
       <c r="K21" s="6" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L21" s="5">
         <f>IF(K21=0,"",(J21-K21)/K21)</f>
         <v/>
       </c>
       <c r="M21" s="6" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="N21" s="6" t="n">
         <v>1</v>
@@ -2394,7 +2394,7 @@
         <v>200</v>
       </c>
       <c r="R21" s="7" t="n">
-        <v>12.49</v>
+        <v>4.38</v>
       </c>
       <c r="S21" s="2">
         <f>IF(AND('Engine Inputs'!E21=0,R21=0),"",IF('Engine Inputs'!E21=0,"📈 Up",IF((R21-'Engine Inputs'!E21)/'Engine Inputs'!E21&gt;Config!$B$2,"📈 Up",IF((R21-'Engine Inputs'!E21)/'Engine Inputs'!E21&lt;-Config!$B$2,"📉 Down","➡ Stable"))))</f>
@@ -2437,7 +2437,7 @@
         </is>
       </c>
       <c r="D22" s="3" t="n">
-        <v>46251</v>
+        <v>46252</v>
       </c>
       <c r="E22" s="10" t="n">
         <v>0</v>
@@ -2526,7 +2526,7 @@
         </is>
       </c>
       <c r="D23" s="3" t="n">
-        <v>46251</v>
+        <v>46252</v>
       </c>
       <c r="E23" s="7" t="n">
         <v>0</v>
@@ -2615,13 +2615,13 @@
         </is>
       </c>
       <c r="D24" s="3" t="n">
-        <v>46251</v>
+        <v>46252</v>
       </c>
       <c r="E24" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="F24" s="7" t="n">
         <v>20.89</v>
-      </c>
-      <c r="F24" s="7" t="n">
-        <v>0</v>
       </c>
       <c r="G24" s="7">
         <f>E24-F24</f>
@@ -2632,23 +2632,23 @@
         <v/>
       </c>
       <c r="I24" s="7" t="n">
-        <v>28.67</v>
+        <v>0</v>
       </c>
       <c r="J24" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="K24" s="6" t="n">
         <v>1</v>
-      </c>
-      <c r="K24" s="6" t="n">
-        <v>0</v>
       </c>
       <c r="L24" s="5">
         <f>IF(K24=0,"",(J24-K24)/K24)</f>
         <v/>
       </c>
       <c r="M24" s="6" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="N24" s="6" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="O24" s="7">
         <f>IF(J24=0,"",E24/J24)</f>
@@ -2661,7 +2661,7 @@
         <v>151</v>
       </c>
       <c r="R24" s="7" t="n">
-        <v>12.89</v>
+        <v>0</v>
       </c>
       <c r="S24" s="2">
         <f>IF(AND('Engine Inputs'!E24=0,R24=0),"",IF('Engine Inputs'!E24=0,"📈 Up",IF((R24-'Engine Inputs'!E24)/'Engine Inputs'!E24&gt;Config!$B$2,"📈 Up",IF((R24-'Engine Inputs'!E24)/'Engine Inputs'!E24&lt;-Config!$B$2,"📉 Down","➡ Stable"))))</f>
@@ -2704,7 +2704,7 @@
         </is>
       </c>
       <c r="D25" s="3" t="n">
-        <v>46251</v>
+        <v>46252</v>
       </c>
       <c r="E25" s="10" t="n">
         <v>0</v>
@@ -2793,7 +2793,7 @@
         </is>
       </c>
       <c r="D26" s="3" t="n">
-        <v>46251</v>
+        <v>46252</v>
       </c>
       <c r="E26" s="7" t="n">
         <v>0</v>
@@ -2882,13 +2882,13 @@
         </is>
       </c>
       <c r="D27" s="3" t="n">
-        <v>46251</v>
+        <v>46252</v>
       </c>
       <c r="E27" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="F27" s="4" t="n">
         <v>17.52</v>
-      </c>
-      <c r="F27" s="4" t="n">
-        <v>12.96</v>
       </c>
       <c r="G27" s="4">
         <f>E27-F27</f>
@@ -2902,7 +2902,7 @@
         <v>0</v>
       </c>
       <c r="J27" s="6" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K27" s="6" t="n">
         <v>1</v>
@@ -2915,7 +2915,7 @@
         <v>0</v>
       </c>
       <c r="N27" s="6" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="O27" s="4">
         <f>IF(J27=0,"",E27/J27)</f>
@@ -2928,7 +2928,7 @@
         <v>65</v>
       </c>
       <c r="R27" s="4" t="n">
-        <v>17.52</v>
+        <v>0</v>
       </c>
       <c r="S27" s="2">
         <f>IF(AND('Engine Inputs'!E27=0,R27=0),"",IF('Engine Inputs'!E27=0,"📈 Up",IF((R27-'Engine Inputs'!E27)/'Engine Inputs'!E27&gt;Config!$B$2,"📈 Up",IF((R27-'Engine Inputs'!E27)/'Engine Inputs'!E27&lt;-Config!$B$2,"📉 Down","➡ Stable"))))</f>
@@ -2971,7 +2971,7 @@
         </is>
       </c>
       <c r="D28" s="3" t="n">
-        <v>46251</v>
+        <v>46252</v>
       </c>
       <c r="E28" s="9" t="n">
         <v>0</v>
@@ -3060,7 +3060,7 @@
         </is>
       </c>
       <c r="D29" s="3" t="n">
-        <v>46251</v>
+        <v>46252</v>
       </c>
       <c r="E29" s="7" t="n">
         <v>0</v>
@@ -3149,7 +3149,7 @@
         </is>
       </c>
       <c r="D30" s="3" t="n">
-        <v>46251</v>
+        <v>46252</v>
       </c>
       <c r="E30" s="7" t="n">
         <v>0</v>
@@ -3238,7 +3238,7 @@
         </is>
       </c>
       <c r="D31" s="3" t="n">
-        <v>46251</v>
+        <v>46252</v>
       </c>
       <c r="E31" s="7" t="n">
         <v>0</v>
@@ -3327,7 +3327,7 @@
         </is>
       </c>
       <c r="D32" s="3" t="n">
-        <v>46251</v>
+        <v>46252</v>
       </c>
       <c r="E32" s="4" t="n">
         <v>0</v>
@@ -3416,7 +3416,7 @@
         </is>
       </c>
       <c r="D33" s="3" t="n">
-        <v>46251</v>
+        <v>46252</v>
       </c>
       <c r="E33" s="7" t="n">
         <v>0</v>
@@ -3521,7 +3521,7 @@
         </is>
       </c>
       <c r="B2" s="12" t="n">
-        <v>46251</v>
+        <v>46252</v>
       </c>
     </row>
     <row r="3">
@@ -3531,7 +3531,7 @@
         </is>
       </c>
       <c r="B3" s="12" t="n">
-        <v>46252</v>
+        <v>46253</v>
       </c>
     </row>
     <row r="5">
@@ -3943,12 +3943,12 @@
       </c>
       <c r="D1" s="13" t="inlineStr">
         <is>
-          <t>PH Sales 2026-08-16</t>
+          <t>PH Sales 2026-08-17</t>
         </is>
       </c>
       <c r="E1" s="13" t="inlineStr">
         <is>
-          <t>AH Sales 2026-08-16</t>
+          <t>AH Sales 2026-08-17</t>
         </is>
       </c>
       <c r="F1" s="15" t="inlineStr">
@@ -3974,10 +3974,10 @@
         </is>
       </c>
       <c r="D2" s="16" t="n">
-        <v>582.95</v>
+        <v>517.77</v>
       </c>
       <c r="E2" s="16" t="n">
-        <v>621.3200000000001</v>
+        <v>591.71</v>
       </c>
     </row>
     <row r="3">
@@ -3997,10 +3997,10 @@
         </is>
       </c>
       <c r="D3" s="16" t="n">
-        <v>157.43</v>
+        <v>183.01</v>
       </c>
       <c r="E3" s="16" t="n">
-        <v>146.03</v>
+        <v>306.32</v>
       </c>
     </row>
     <row r="4">
@@ -4020,10 +4020,10 @@
         </is>
       </c>
       <c r="D4" s="17" t="n">
-        <v>22.44</v>
+        <v>3.78</v>
       </c>
       <c r="E4" s="17" t="n">
-        <v>201.31</v>
+        <v>199.69</v>
       </c>
     </row>
     <row r="5">
@@ -4043,10 +4043,10 @@
         </is>
       </c>
       <c r="D5" s="16" t="n">
-        <v>130.93</v>
+        <v>87.39</v>
       </c>
       <c r="E5" s="16" t="n">
-        <v>106.36</v>
+        <v>234.1</v>
       </c>
     </row>
     <row r="6">
@@ -4066,10 +4066,10 @@
         </is>
       </c>
       <c r="D6" s="17" t="n">
-        <v>0</v>
+        <v>14.99</v>
       </c>
       <c r="E6" s="17" t="n">
-        <v>186.49</v>
+        <v>128.94</v>
       </c>
     </row>
     <row r="7">
@@ -4138,7 +4138,7 @@
         <v>0</v>
       </c>
       <c r="E9" s="16" t="n">
-        <v>197.39</v>
+        <v>223.61</v>
       </c>
     </row>
     <row r="10">
@@ -4158,10 +4158,10 @@
         </is>
       </c>
       <c r="D10" s="17" t="n">
-        <v>58.87</v>
+        <v>37.27</v>
       </c>
       <c r="E10" s="17" t="n">
-        <v>204.99</v>
+        <v>207.36</v>
       </c>
     </row>
     <row r="11">
@@ -4184,7 +4184,7 @@
         <v>0</v>
       </c>
       <c r="E11" s="16" t="n">
-        <v>85.44</v>
+        <v>115.44</v>
       </c>
     </row>
     <row r="12">
@@ -4207,7 +4207,7 @@
         <v>0</v>
       </c>
       <c r="E12" s="17" t="n">
-        <v>33.68</v>
+        <v>7.47</v>
       </c>
     </row>
     <row r="13">
@@ -4230,7 +4230,7 @@
         <v>0</v>
       </c>
       <c r="E13" s="16" t="n">
-        <v>107.38</v>
+        <v>6.99</v>
       </c>
     </row>
     <row r="14">
@@ -4253,7 +4253,7 @@
         <v>0</v>
       </c>
       <c r="E14" s="16" t="n">
-        <v>14.7</v>
+        <v>90.76000000000001</v>
       </c>
     </row>
     <row r="15">
@@ -4276,7 +4276,7 @@
         <v>0</v>
       </c>
       <c r="E15" s="17" t="n">
-        <v>9.41</v>
+        <v>0</v>
       </c>
     </row>
     <row r="16">
@@ -4322,7 +4322,7 @@
         <v>0</v>
       </c>
       <c r="E17" s="18" t="n">
-        <v>14.3</v>
+        <v>26.99</v>
       </c>
     </row>
     <row r="18">
@@ -4345,7 +4345,7 @@
         <v>0</v>
       </c>
       <c r="E18" s="18" t="n">
-        <v>134.96</v>
+        <v>21.5</v>
       </c>
     </row>
     <row r="19">
@@ -4391,7 +4391,7 @@
         <v>0</v>
       </c>
       <c r="E20" s="16" t="n">
-        <v>0</v>
+        <v>34.88</v>
       </c>
     </row>
     <row r="21">
@@ -4414,7 +4414,7 @@
         <v>0</v>
       </c>
       <c r="E21" s="17" t="n">
-        <v>0</v>
+        <v>12.49</v>
       </c>
     </row>
     <row r="22">
@@ -4483,7 +4483,7 @@
         <v>0</v>
       </c>
       <c r="E24" s="17" t="n">
-        <v>0</v>
+        <v>12.89</v>
       </c>
     </row>
     <row r="25">
@@ -4552,7 +4552,7 @@
         <v>0</v>
       </c>
       <c r="E27" s="16" t="n">
-        <v>12.96</v>
+        <v>17.52</v>
       </c>
     </row>
     <row r="28">
@@ -4806,7 +4806,7 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t xml:space="preserve">  Generated 2026-08-18.  "Today" = 2026-08-17.  "Yesterday" = 2026-08-16.  Same Day LY = 2025-08-17.</t>
+          <t xml:space="preserve">  Generated 2026-08-19.  "Today" = 2026-08-18.  "Yesterday" = 2026-08-17.  Same Day LY = 2025-08-18.</t>
         </is>
       </c>
     </row>
@@ -4851,7 +4851,7 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t xml:space="preserve">  Why not 'Completed' only: orders reach Completed about 2 days after purchase. On 2026-08-17</t>
+          <t xml:space="preserve">  Why not 'Completed' only: orders reach Completed about 2 days after purchase. On 2026-08-18</t>
         </is>
       </c>
     </row>
@@ -5162,7 +5162,7 @@
     <row r="72">
       <c r="A72" t="inlineStr">
         <is>
-          <t xml:space="preserve">  (2026-08-17 was a Monday; 2025-08-17 was a Sunday). Day-of-week effects are present in this comparison.</t>
+          <t xml:space="preserve">  (2026-08-18 was a Tuesday; 2025-08-18 was a Monday). Day-of-week effects are present in this comparison.</t>
         </is>
       </c>
     </row>

</xml_diff>